<commit_message>
Update dashboard and Excel files - 26-05-2026 15:39:19.57
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q75"/>
+  <dimension ref="A1:Q86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6095,6 +6095,831 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-05-25 09:43:36</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>23946.5</v>
+      </c>
+      <c r="F76" t="n">
+        <v>23973.2</v>
+      </c>
+      <c r="G76" t="n">
+        <v>23879.8</v>
+      </c>
+      <c r="H76" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I76" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>2026-05-25 10:09:50</t>
+        </is>
+      </c>
+      <c r="K76" t="n">
+        <v>23974</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>-27.5</v>
+      </c>
+      <c r="N76" t="n">
+        <v>-2062.5</v>
+      </c>
+      <c r="O76" t="n">
+        <v>4</v>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.76 → 0.76 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23950: CE 5m +1,176,175 | PE 5m -734,630 | OTM CE +1,852,955 | OTM PE +253,825
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-05-25 10:26:20</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>23975.5</v>
+      </c>
+      <c r="F77" t="n">
+        <v>23948.8</v>
+      </c>
+      <c r="G77" t="n">
+        <v>24042.2</v>
+      </c>
+      <c r="H77" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I77" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>2026-05-25 10:32:08</t>
+        </is>
+      </c>
+      <c r="K77" t="n">
+        <v>23988</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M77" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="N77" t="n">
+        <v>937.5</v>
+      </c>
+      <c r="O77" t="n">
+        <v>4</v>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.88 → 0.88 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23950: CE 5m -561,080 | PE 5m +530,205 | OTM CE -358,865 | OTM PE +525,850
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (20.5x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-05-25 10:32:09</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>23988</v>
+      </c>
+      <c r="F78" t="n">
+        <v>24014.7</v>
+      </c>
+      <c r="G78" t="n">
+        <v>23921.3</v>
+      </c>
+      <c r="H78" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I78" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>2026-05-25 10:49:19</t>
+        </is>
+      </c>
+      <c r="K78" t="n">
+        <v>24005</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>-17</v>
+      </c>
+      <c r="N78" t="n">
+        <v>-1275</v>
+      </c>
+      <c r="O78" t="n">
+        <v>4</v>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.90 → 0.89 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23950: CE 5m +386,815 | PE 5m +167,765 | OTM CE +434,330 | OTM PE +45,500
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-05-25 10:49:19</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>24006.9</v>
+      </c>
+      <c r="F79" t="n">
+        <v>23980.2</v>
+      </c>
+      <c r="G79" t="n">
+        <v>24073.6</v>
+      </c>
+      <c r="H79" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I79" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>2026-05-25 11:02:40</t>
+        </is>
+      </c>
+      <c r="K79" t="n">
+        <v>23979</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M79" t="n">
+        <v>-27.9</v>
+      </c>
+      <c r="N79" t="n">
+        <v>-2092.5</v>
+      </c>
+      <c r="O79" t="n">
+        <v>4</v>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.89 → 0.90 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 24000: CE 5m +383,240 | PE 5m +868,335 | OTM CE +24,050 | OTM PE +355,810
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (31.6x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-05-26 10:23:57</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>24060</v>
+      </c>
+      <c r="F80" t="n">
+        <v>24086.7</v>
+      </c>
+      <c r="G80" t="n">
+        <v>23993.3</v>
+      </c>
+      <c r="H80" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I80" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>2026-05-26 11:05:30</t>
+        </is>
+      </c>
+      <c r="K80" t="n">
+        <v>24070</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M80" t="n">
+        <v>-10</v>
+      </c>
+      <c r="N80" t="n">
+        <v>-750</v>
+      </c>
+      <c r="O80" t="n">
+        <v>4</v>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.14 → 1.13 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 24050: CE 5m +569,140 | PE 5m +182,195 | OTM CE +736,775 | OTM PE +352,690
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-05-26 11:05:31</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>24074</v>
+      </c>
+      <c r="F81" t="n">
+        <v>24047.3</v>
+      </c>
+      <c r="G81" t="n">
+        <v>24140.7</v>
+      </c>
+      <c r="H81" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I81" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>2026-05-26 11:20:49</t>
+        </is>
+      </c>
+      <c r="K81" t="n">
+        <v>24063.5</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="N81" t="n">
+        <v>-787.5</v>
+      </c>
+      <c r="O81" t="n">
+        <v>4</v>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 1.21 → 1.22 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 24100: CE 5m -350,545 | PE 5m +705,445 | OTM CE +167,635 | OTM PE +1,014,000
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (24.8x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-05-26 11:20:50</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>24063.5</v>
+      </c>
+      <c r="F82" t="n">
+        <v>24090.2</v>
+      </c>
+      <c r="G82" t="n">
+        <v>23996.8</v>
+      </c>
+      <c r="H82" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I82" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>2026-05-26 12:45:53</t>
+        </is>
+      </c>
+      <c r="K82" t="n">
+        <v>23993.9</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="N82" t="n">
+        <v>5220</v>
+      </c>
+      <c r="O82" t="n">
+        <v>4</v>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.29 → 1.28 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 24050: CE 5m +655,980 | PE 5m -438,685 | OTM CE +651,105 | OTM PE +287,625
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-05-26 12:50:16</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>23995</v>
+      </c>
+      <c r="F83" t="n">
+        <v>24021.7</v>
+      </c>
+      <c r="G83" t="n">
+        <v>23928.3</v>
+      </c>
+      <c r="H83" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I83" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>2026-05-26 13:26:30</t>
+        </is>
+      </c>
+      <c r="K83" t="n">
+        <v>23977.5</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M83" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="N83" t="n">
+        <v>1312.5</v>
+      </c>
+      <c r="O83" t="n">
+        <v>4</v>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.99 → 0.99 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 24000: CE 5m +3,874,780 | PE 5m -3,442,725 | OTM CE +388,635 | OTM PE +770,510
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-05-26 13:26:31</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>23976</v>
+      </c>
+      <c r="F84" t="n">
+        <v>23949.3</v>
+      </c>
+      <c r="G84" t="n">
+        <v>24042.7</v>
+      </c>
+      <c r="H84" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I84" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>2026-05-26 13:32:48</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>23976.1</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M84" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N84" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="O84" t="n">
+        <v>4</v>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.81 → 0.81 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 24000: CE 5m -615,615 | PE 5m +1,514,565 | OTM CE +223,405 | OTM PE +2,133,040
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (37.2x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-05-26 13:32:48</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>23980</v>
+      </c>
+      <c r="F85" t="n">
+        <v>24006.7</v>
+      </c>
+      <c r="G85" t="n">
+        <v>23913.3</v>
+      </c>
+      <c r="H85" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I85" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>2026-05-26 14:04:14</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
+        <v>23911</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M85" t="n">
+        <v>69</v>
+      </c>
+      <c r="N85" t="n">
+        <v>5175</v>
+      </c>
+      <c r="O85" t="n">
+        <v>4</v>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.80 → 0.80 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 24000: CE 5m +2,038,465 | PE 5m -181,610 | OTM CE +289,705 | OTM PE -836,550
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-05-26 14:55:48</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>23883.1</v>
+      </c>
+      <c r="F86" t="n">
+        <v>23909.8</v>
+      </c>
+      <c r="G86" t="n">
+        <v>23816.4</v>
+      </c>
+      <c r="H86" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I86" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>2026-05-26 14:57:47</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
+        <v>23910</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M86" t="n">
+        <v>-26.9</v>
+      </c>
+      <c r="N86" t="n">
+        <v>-2017.5</v>
+      </c>
+      <c r="O86" t="n">
+        <v>4</v>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.88 → 0.86 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23900: CE 5m +5,197,725 | PE 5m -9,220,380 | OTM CE -5,337,280 | OTM PE +2,168,790
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6106,10 +6931,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
@@ -7984,6 +8809,899 @@
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>90</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-05-25 11:05:51</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>23998</v>
+      </c>
+      <c r="H40" t="n">
+        <v>24024.7</v>
+      </c>
+      <c r="I40" t="n">
+        <v>23931.3</v>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>91</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-05-25 11:13:06</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>23998</v>
+      </c>
+      <c r="H41" t="n">
+        <v>23971.3</v>
+      </c>
+      <c r="I41" t="n">
+        <v>24064.7</v>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>92</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-05-25 11:17:43</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>23995</v>
+      </c>
+      <c r="H42" t="n">
+        <v>23968.3</v>
+      </c>
+      <c r="I42" t="n">
+        <v>24061.7</v>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>93</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-05-25 11:35:04</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>23980</v>
+      </c>
+      <c r="H43" t="n">
+        <v>24006.7</v>
+      </c>
+      <c r="I43" t="n">
+        <v>23913.3</v>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>94</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-05-25 11:41:57</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>4</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>23996.7</v>
+      </c>
+      <c r="H44" t="n">
+        <v>24023.4</v>
+      </c>
+      <c r="I44" t="n">
+        <v>23930</v>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>95</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-05-25 11:42:52</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>4</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>24000</v>
+      </c>
+      <c r="H45" t="n">
+        <v>24026.7</v>
+      </c>
+      <c r="I45" t="n">
+        <v>23933.3</v>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>96</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:12:34</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>4</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>23976</v>
+      </c>
+      <c r="H46" t="n">
+        <v>24002.7</v>
+      </c>
+      <c r="I46" t="n">
+        <v>23909.3</v>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>97</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:14:36</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>4</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>23974</v>
+      </c>
+      <c r="H47" t="n">
+        <v>24000.7</v>
+      </c>
+      <c r="I47" t="n">
+        <v>23907.3</v>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>98</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:20:04</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>4</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>23973</v>
+      </c>
+      <c r="H48" t="n">
+        <v>23999.7</v>
+      </c>
+      <c r="I48" t="n">
+        <v>23906.3</v>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>99</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:47:10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>23960</v>
+      </c>
+      <c r="H49" t="n">
+        <v>23986.7</v>
+      </c>
+      <c r="I49" t="n">
+        <v>23893.3</v>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>100</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-05-25 13:48:08</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>4</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>23985</v>
+      </c>
+      <c r="H50" t="n">
+        <v>24011.7</v>
+      </c>
+      <c r="I50" t="n">
+        <v>23918.3</v>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>101</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:06:01</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>23989.9</v>
+      </c>
+      <c r="H51" t="n">
+        <v>24016.6</v>
+      </c>
+      <c r="I51" t="n">
+        <v>23923.2</v>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>102</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:09:54</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>4</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>23973</v>
+      </c>
+      <c r="H52" t="n">
+        <v>23999.7</v>
+      </c>
+      <c r="I52" t="n">
+        <v>23906.3</v>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>103</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:11:01</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>4</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>23975</v>
+      </c>
+      <c r="H53" t="n">
+        <v>24001.7</v>
+      </c>
+      <c r="I53" t="n">
+        <v>23908.3</v>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>104</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:27:32</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>4</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>23992</v>
+      </c>
+      <c r="H54" t="n">
+        <v>24018.7</v>
+      </c>
+      <c r="I54" t="n">
+        <v>23925.3</v>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>105</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:46:14</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>4</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>24036</v>
+      </c>
+      <c r="H55" t="n">
+        <v>24009.3</v>
+      </c>
+      <c r="I55" t="n">
+        <v>24102.7</v>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>106</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:46:41</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>4</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>24037.9</v>
+      </c>
+      <c r="H56" t="n">
+        <v>24011.2</v>
+      </c>
+      <c r="I56" t="n">
+        <v>24104.6</v>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>107</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:51:47</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>4</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>24047.9</v>
+      </c>
+      <c r="H57" t="n">
+        <v>24021.2</v>
+      </c>
+      <c r="I57" t="n">
+        <v>24114.6</v>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>108</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:51:59</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>4</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>24045.6</v>
+      </c>
+      <c r="H58" t="n">
+        <v>24018.9</v>
+      </c>
+      <c r="I58" t="n">
+        <v>24112.3</v>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr">
         <is>
           <t>TRACKING</t>
         </is>
@@ -8026,7 +9744,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3">
@@ -8036,7 +9754,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -8046,7 +9764,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -8057,7 +9775,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35.14%</t>
+          <t>36.47%</t>
         </is>
       </c>
     </row>
@@ -8069,7 +9787,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 15,832.50</t>
+          <t>Rs. 19,500.00</t>
         </is>
       </c>
     </row>
@@ -8081,7 +9799,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>211.10</t>
+          <t>260.00</t>
         </is>
       </c>
     </row>
@@ -8093,7 +9811,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs. 4,274.71</t>
+          <t>Rs. 3,993.39</t>
         </is>
       </c>
     </row>
@@ -8105,7 +9823,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -1,985.62</t>
+          <t>Rs. -1,931.39</t>
         </is>
       </c>
     </row>
@@ -8141,7 +9859,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.19</t>
         </is>
       </c>
     </row>
@@ -8152,7 +9870,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>38</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14">
@@ -8163,7 +9881,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-22 16:43:06</t>
+          <t>2026-05-26 15:39:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 01-06-2026 12:43:29.54
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q86"/>
+  <dimension ref="A1:Q95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6920,6 +6920,681 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-05-29 11:14:23</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>24000.2</v>
+      </c>
+      <c r="F87" t="n">
+        <v>23973.5</v>
+      </c>
+      <c r="G87" t="n">
+        <v>24066.9</v>
+      </c>
+      <c r="H87" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I87" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>2026-05-29 11:14:25</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
+        <v>23913</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M87" t="n">
+        <v>-87.2</v>
+      </c>
+      <c r="N87" t="n">
+        <v>-6540</v>
+      </c>
+      <c r="O87" t="n">
+        <v>4</v>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.82 → 0.82 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23900: CE 5m -229,125 | PE 5m +648,635 | OTM CE -143,455 | OTM PE +221,195
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (22.2x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-05-29 13:07:26</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>23910</v>
+      </c>
+      <c r="F88" t="n">
+        <v>23936.7</v>
+      </c>
+      <c r="G88" t="n">
+        <v>23843.3</v>
+      </c>
+      <c r="H88" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I88" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2026-05-29 14:56:03</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>23913</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M88" t="n">
+        <v>-3</v>
+      </c>
+      <c r="N88" t="n">
+        <v>-225</v>
+      </c>
+      <c r="O88" t="n">
+        <v>4</v>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.82 → 0.81 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23800: CE 5m +464,620 | PE 5m -150,995 | OTM CE +316,745 | OTM PE -39,000
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-05-29 14:56:04</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>23840</v>
+      </c>
+      <c r="F89" t="n">
+        <v>23813.3</v>
+      </c>
+      <c r="G89" t="n">
+        <v>23906.7</v>
+      </c>
+      <c r="H89" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I89" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>2026-05-29 14:56:05</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>23913</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M89" t="n">
+        <v>73</v>
+      </c>
+      <c r="N89" t="n">
+        <v>5475</v>
+      </c>
+      <c r="O89" t="n">
+        <v>4</v>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.76 → 0.76 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23750: CE 5m -52,780 | PE 5m -61,165 | OTM CE -223,665 | OTM PE -10,010
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (29.1x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-05-29 15:04:06</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26MAYFUT</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>23727.4</v>
+      </c>
+      <c r="F90" t="n">
+        <v>23754.1</v>
+      </c>
+      <c r="G90" t="n">
+        <v>23660.7</v>
+      </c>
+      <c r="H90" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I90" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>2026-05-29 15:04:07</t>
+        </is>
+      </c>
+      <c r="K90" t="n">
+        <v>23913</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>-185.6</v>
+      </c>
+      <c r="N90" t="n">
+        <v>-13920</v>
+      </c>
+      <c r="O90" t="n">
+        <v>4</v>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.97 → 0.95 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23600: CE 5m +810,485 | PE 5m -225,875 | OTM CE +632,515 | OTM PE +427,570
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-06-01 10:57:03</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>23661.5</v>
+      </c>
+      <c r="F91" t="n">
+        <v>23634.8</v>
+      </c>
+      <c r="G91" t="n">
+        <v>23728.2</v>
+      </c>
+      <c r="H91" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I91" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:29:52</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>23632</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M91" t="n">
+        <v>-29.5</v>
+      </c>
+      <c r="N91" t="n">
+        <v>-2212.5</v>
+      </c>
+      <c r="O91" t="n">
+        <v>4</v>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.73 → 0.74 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23600: CE 5m -912,470 | PE 5m +1,203,540 | OTM CE -544,310 | OTM PE +350,090
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (24.3x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:36:17</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>23624.9</v>
+      </c>
+      <c r="F92" t="n">
+        <v>23651.6</v>
+      </c>
+      <c r="G92" t="n">
+        <v>23558.2</v>
+      </c>
+      <c r="H92" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I92" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:59:27</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>23558</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M92" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="N92" t="n">
+        <v>5017.5</v>
+      </c>
+      <c r="O92" t="n">
+        <v>4</v>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.86 → 0.85 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23550: CE 5m +962,715 | PE 5m -1,097,980 | OTM CE +1,618,110 | OTM PE -338,260
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:03:47</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>23560</v>
+      </c>
+      <c r="F93" t="n">
+        <v>23586.7</v>
+      </c>
+      <c r="G93" t="n">
+        <v>23493.3</v>
+      </c>
+      <c r="H93" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I93" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:14:22</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>23587.7</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M93" t="n">
+        <v>-27.7</v>
+      </c>
+      <c r="N93" t="n">
+        <v>-2077.5</v>
+      </c>
+      <c r="O93" t="n">
+        <v>4</v>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.78 → 0.78 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23500: CE 5m +2,417,610 | PE 5m -2,857,140 | OTM CE +1,404,195 | OTM PE -181,610
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:17:34</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>23578.5</v>
+      </c>
+      <c r="F94" t="n">
+        <v>23551.8</v>
+      </c>
+      <c r="G94" t="n">
+        <v>23645.2</v>
+      </c>
+      <c r="H94" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I94" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:34:30</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>23570</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M94" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="N94" t="n">
+        <v>-637.5</v>
+      </c>
+      <c r="O94" t="n">
+        <v>4</v>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.67 → 0.69 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23500: CE 5m -620,295 | PE 5m +913,900 | OTM CE +97,630 | OTM PE +44,395
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (50.4x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:34:32</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>23571</v>
+      </c>
+      <c r="F95" t="n">
+        <v>23597.7</v>
+      </c>
+      <c r="G95" t="n">
+        <v>23504.3</v>
+      </c>
+      <c r="H95" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I95" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:43:05</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>23570.5</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M95" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N95" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="O95" t="n">
+        <v>4</v>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.83 → 0.83 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23500: CE 5m +153,725 | PE 5m +252,200 | OTM CE +90,545 | OTM PE +78,715
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6931,7 +7606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9707,6 +10382,100 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>109</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:34:41</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>4</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>23572</v>
+      </c>
+      <c r="H59" t="n">
+        <v>23598.7</v>
+      </c>
+      <c r="I59" t="n">
+        <v>23505.3</v>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>110</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:42:59</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>4</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>23568.3</v>
+      </c>
+      <c r="H60" t="n">
+        <v>23541.6</v>
+      </c>
+      <c r="I60" t="n">
+        <v>23635</v>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9744,7 +10513,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
@@ -9754,7 +10523,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -9764,7 +10533,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
@@ -9775,7 +10544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>36.47%</t>
+          <t>36.17%</t>
         </is>
       </c>
     </row>
@@ -9787,7 +10556,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 19,500.00</t>
+          <t>Rs. 4,417.50</t>
         </is>
       </c>
     </row>
@@ -9799,7 +10568,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>260.00</t>
+          <t>58.90</t>
         </is>
       </c>
     </row>
@@ -9811,7 +10580,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs. 3,993.39</t>
+          <t>Rs. 3,950.74</t>
         </is>
       </c>
     </row>
@@ -9823,7 +10592,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -1,931.39</t>
+          <t>Rs. -2,165.12</t>
         </is>
       </c>
     </row>
@@ -9847,7 +10616,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rs. -2,362.50</t>
+          <t>Rs. -13,920.00</t>
         </is>
       </c>
     </row>
@@ -9859,7 +10628,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.03</t>
         </is>
       </c>
     </row>
@@ -9870,7 +10639,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14">
@@ -9881,7 +10650,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-26 15:39:18</t>
+          <t>2026-06-01 12:43:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 01-06-2026 14:08:33.18
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q95"/>
+  <dimension ref="A1:Q96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -7595,6 +7595,81 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-06-01 12:43:06</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>23570.5</v>
+      </c>
+      <c r="F96" t="n">
+        <v>23543.8</v>
+      </c>
+      <c r="G96" t="n">
+        <v>23637.2</v>
+      </c>
+      <c r="H96" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="I96" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>2026-06-01 13:08:10</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>23543.5</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M96" t="n">
+        <v>-27</v>
+      </c>
+      <c r="N96" t="n">
+        <v>-2025</v>
+      </c>
+      <c r="O96" t="n">
+        <v>4</v>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.83 → 0.83 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23500: CE 5m -24,180 | PE 5m +149,240 | OTM CE +40,430 | OTM PE -62,400
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (21.7x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7606,7 +7681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10384,16 +10459,16 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-06-01 12:34:41</t>
+          <t>2026-06-01 12:42:59</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -10406,17 +10481,17 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>23572</v>
+        <v>23568.3</v>
       </c>
       <c r="H59" t="n">
-        <v>23598.7</v>
+        <v>23541.6</v>
       </c>
       <c r="I59" t="n">
-        <v>23505.3</v>
+        <v>23635</v>
       </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
@@ -10431,16 +10506,16 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-06-01 12:42:59</t>
+          <t>2026-06-01 13:10:52</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -10453,17 +10528,17 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>BULLISH</t>
+          <t>BEARISH</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>23568.3</v>
+        <v>23532.9</v>
       </c>
       <c r="H60" t="n">
-        <v>23541.6</v>
+        <v>23559.6</v>
       </c>
       <c r="I60" t="n">
-        <v>23635</v>
+        <v>23466.2</v>
       </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
@@ -10471,6 +10546,241 @@
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>112</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:03:44</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>23501.8</v>
+      </c>
+      <c r="H61" t="n">
+        <v>23528.5</v>
+      </c>
+      <c r="I61" t="n">
+        <v>23435.1</v>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>113</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:04:43</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>23501.5</v>
+      </c>
+      <c r="H62" t="n">
+        <v>23528.2</v>
+      </c>
+      <c r="I62" t="n">
+        <v>23434.8</v>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>114</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:05:07</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>4</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>23504.4</v>
+      </c>
+      <c r="H63" t="n">
+        <v>23531.1</v>
+      </c>
+      <c r="I63" t="n">
+        <v>23437.7</v>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>115</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:05:29</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>4</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>23497.2</v>
+      </c>
+      <c r="H64" t="n">
+        <v>23523.9</v>
+      </c>
+      <c r="I64" t="n">
+        <v>23430.5</v>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>116</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:05:58</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>23505</v>
+      </c>
+      <c r="H65" t="n">
+        <v>23531.7</v>
+      </c>
+      <c r="I65" t="n">
+        <v>23438.3</v>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr">
         <is>
           <t>TRACKING</t>
         </is>
@@ -10513,7 +10823,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -10533,7 +10843,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -10544,7 +10854,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>36.17%</t>
+          <t>35.79%</t>
         </is>
       </c>
     </row>
@@ -10556,7 +10866,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 4,417.50</t>
+          <t>Rs. 2,392.50</t>
         </is>
       </c>
     </row>
@@ -10568,7 +10878,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>58.90</t>
+          <t>31.90</t>
         </is>
       </c>
     </row>
@@ -10592,7 +10902,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -2,165.12</t>
+          <t>Rs. -2,162.83</t>
         </is>
       </c>
     </row>
@@ -10628,7 +10938,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.02</t>
         </is>
       </c>
     </row>
@@ -10639,7 +10949,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14">
@@ -10650,7 +10960,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-01 12:43:29</t>
+          <t>2026-06-01 14:08:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 05-06-2026 14:53:36.51
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,10 +427,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q96"/>
+  <dimension ref="A1:Q114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -7670,6 +7670,1356 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-06-03 09:47:46</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>23334</v>
+      </c>
+      <c r="F97" t="n">
+        <v>23400.7</v>
+      </c>
+      <c r="G97" t="n">
+        <v>23267.3</v>
+      </c>
+      <c r="H97" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I97" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:09:15</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>23264.5</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M97" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="N97" t="n">
+        <v>5212.5</v>
+      </c>
+      <c r="O97" t="n">
+        <v>4</v>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.98 → 0.97 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23250: CE 5m +152,295 | PE 5m +106,795 | OTM CE +438,100 | OTM PE +63,765
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:09:46</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>23262</v>
+      </c>
+      <c r="F98" t="n">
+        <v>23328.7</v>
+      </c>
+      <c r="G98" t="n">
+        <v>23195.3</v>
+      </c>
+      <c r="H98" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I98" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>2026-06-03 12:30:40</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>23330</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M98" t="n">
+        <v>-68</v>
+      </c>
+      <c r="N98" t="n">
+        <v>-5100</v>
+      </c>
+      <c r="O98" t="n">
+        <v>4</v>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 0.93 → 0.92 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23200: CE 5m +111,020 | PE 5m +60,255 | OTM CE +113,295 | OTM PE +110,565
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-06-03 12:35:25</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>23370</v>
+      </c>
+      <c r="F99" t="n">
+        <v>23303.3</v>
+      </c>
+      <c r="G99" t="n">
+        <v>23436.7</v>
+      </c>
+      <c r="H99" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I99" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>2026-06-03 12:53:51</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>23375.1</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M99" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="N99" t="n">
+        <v>382.5</v>
+      </c>
+      <c r="O99" t="n">
+        <v>4</v>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.79 → 0.81 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23300: CE 5m -1,114,165 | PE 5m +711,360 | OTM CE -531,570 | OTM PE +150,865
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (33.4x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-06-03 12:53:51</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>23375.1</v>
+      </c>
+      <c r="F100" t="n">
+        <v>23441.8</v>
+      </c>
+      <c r="G100" t="n">
+        <v>23308.4</v>
+      </c>
+      <c r="H100" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I100" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:15:38</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>23392</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M100" t="n">
+        <v>-16.9</v>
+      </c>
+      <c r="N100" t="n">
+        <v>-1267.5</v>
+      </c>
+      <c r="O100" t="n">
+        <v>4</v>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.03 → 1.03 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23300: CE 5m +307,840 | PE 5m -92,820 | OTM CE +102,960 | OTM PE -4,680
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:15:39</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>23389.3</v>
+      </c>
+      <c r="F101" t="n">
+        <v>23322.6</v>
+      </c>
+      <c r="G101" t="n">
+        <v>23456</v>
+      </c>
+      <c r="H101" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I101" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:46:56</t>
+        </is>
+      </c>
+      <c r="K101" t="n">
+        <v>23456.5</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M101" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="N101" t="n">
+        <v>5040</v>
+      </c>
+      <c r="O101" t="n">
+        <v>4</v>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.98 → 0.99 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23300: CE 5m -182,195 | PE 5m -132,665 | OTM CE -74,100 | OTM PE +43,680
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (50.7x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:02:50</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>23480.8</v>
+      </c>
+      <c r="F102" t="n">
+        <v>23547.5</v>
+      </c>
+      <c r="G102" t="n">
+        <v>23414.1</v>
+      </c>
+      <c r="H102" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I102" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:23:04</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>23549</v>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M102" t="n">
+        <v>-68.2</v>
+      </c>
+      <c r="N102" t="n">
+        <v>-5115</v>
+      </c>
+      <c r="O102" t="n">
+        <v>4</v>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.12 → 1.02 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23400: CE 5m +184,535 | PE 5m -131,040 | OTM CE +72,540 | OTM PE -41,600
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-06-04 09:33:54</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>23405.9</v>
+      </c>
+      <c r="F103" t="n">
+        <v>23472.6</v>
+      </c>
+      <c r="G103" t="n">
+        <v>23339.2</v>
+      </c>
+      <c r="H103" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I103" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>2026-06-04 09:41:05</t>
+        </is>
+      </c>
+      <c r="K103" t="n">
+        <v>23380.1</v>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M103" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="N103" t="n">
+        <v>1935</v>
+      </c>
+      <c r="O103" t="n">
+        <v>4</v>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.16 → 1.15 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23350: CE 5m +283,725 | PE 5m +122,200 | OTM CE +186,745 | OTM PE +60,255
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-06-04 09:41:05</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>23381.3</v>
+      </c>
+      <c r="F104" t="n">
+        <v>23314.6</v>
+      </c>
+      <c r="G104" t="n">
+        <v>23448</v>
+      </c>
+      <c r="H104" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I104" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>2026-06-04 09:49:03</t>
+        </is>
+      </c>
+      <c r="K104" t="n">
+        <v>23449</v>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M104" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="N104" t="n">
+        <v>5077.5</v>
+      </c>
+      <c r="O104" t="n">
+        <v>4</v>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 1.16 → 1.26 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23300: CE 5m -66,560 | PE 5m +206,570 | OTM CE -47,450 | OTM PE -50,960
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (33.2x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-06-04 10:30:20</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>23490</v>
+      </c>
+      <c r="F105" t="n">
+        <v>23423.3</v>
+      </c>
+      <c r="G105" t="n">
+        <v>23556.7</v>
+      </c>
+      <c r="H105" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I105" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>2026-06-04 10:33:40</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>23460</v>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M105" t="n">
+        <v>-30</v>
+      </c>
+      <c r="N105" t="n">
+        <v>-2250</v>
+      </c>
+      <c r="O105" t="n">
+        <v>4</v>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 1.23 → 1.34 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23400: CE 5m -155,480 | PE 5m +71,305 | OTM CE -10,985 | OTM PE +87,295
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (21.8x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-06-04 10:33:41</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>23462.6</v>
+      </c>
+      <c r="F106" t="n">
+        <v>23529.3</v>
+      </c>
+      <c r="G106" t="n">
+        <v>23395.9</v>
+      </c>
+      <c r="H106" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I106" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>2026-06-04 10:51:08</t>
+        </is>
+      </c>
+      <c r="K106" t="n">
+        <v>23481</v>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M106" t="n">
+        <v>-18.4</v>
+      </c>
+      <c r="N106" t="n">
+        <v>-1380</v>
+      </c>
+      <c r="O106" t="n">
+        <v>4</v>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.33 → 1.33 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23400: CE 5m -70,590 | PE 5m -42,445 | OTM CE +14,495 | OTM PE -71,695
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-06-04 10:51:09</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>23481</v>
+      </c>
+      <c r="F107" t="n">
+        <v>23414.3</v>
+      </c>
+      <c r="G107" t="n">
+        <v>23547.7</v>
+      </c>
+      <c r="H107" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I107" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:32:16</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>23413.2</v>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M107" t="n">
+        <v>-67.8</v>
+      </c>
+      <c r="N107" t="n">
+        <v>-5085</v>
+      </c>
+      <c r="O107" t="n">
+        <v>4</v>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 1.22 → 1.22 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23400: CE 5m -281,580 | PE 5m +62,855 | OTM CE +100,230 | OTM PE -97,500
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (23.9x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-06-05 09:54:05</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>23538.3</v>
+      </c>
+      <c r="F108" t="n">
+        <v>23605</v>
+      </c>
+      <c r="G108" t="n">
+        <v>23471.6</v>
+      </c>
+      <c r="H108" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I108" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>2026-06-05 10:10:37</t>
+        </is>
+      </c>
+      <c r="K108" t="n">
+        <v>23569</v>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M108" t="n">
+        <v>-30.7</v>
+      </c>
+      <c r="N108" t="n">
+        <v>-2302.5</v>
+      </c>
+      <c r="O108" t="n">
+        <v>4</v>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.11 → 1.10 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23450: CE 5m +651,950 | PE 5m -241,540 | OTM CE +1,077,765 | OTM PE +13,650
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.7x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-06-05 10:10:38</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>23559.9</v>
+      </c>
+      <c r="F109" t="n">
+        <v>23493.2</v>
+      </c>
+      <c r="G109" t="n">
+        <v>23626.6</v>
+      </c>
+      <c r="H109" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I109" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>2026-06-05 10:17:53</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>23560</v>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M109" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N109" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="O109" t="n">
+        <v>4</v>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.86 → 0.89 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23500: CE 5m +238,095 | PE 5m +1,109,160 | OTM CE +60,775 | OTM PE +624,195
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (22.9x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-06-05 10:17:54</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>23545</v>
+      </c>
+      <c r="F110" t="n">
+        <v>23611.7</v>
+      </c>
+      <c r="G110" t="n">
+        <v>23478.3</v>
+      </c>
+      <c r="H110" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I110" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>2026-06-05 10:36:10</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>23476</v>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M110" t="n">
+        <v>69</v>
+      </c>
+      <c r="N110" t="n">
+        <v>5175</v>
+      </c>
+      <c r="O110" t="n">
+        <v>4</v>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.22 → 1.19 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23500: CE 5m +811,135 | PE 5m -183,365 | OTM CE +338,650 | OTM PE -295,165
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-06-05 10:38:26</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>23464</v>
+      </c>
+      <c r="F111" t="n">
+        <v>23530.7</v>
+      </c>
+      <c r="G111" t="n">
+        <v>23397.3</v>
+      </c>
+      <c r="H111" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I111" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:02:12</t>
+        </is>
+      </c>
+      <c r="K111" t="n">
+        <v>23480</v>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M111" t="n">
+        <v>-16</v>
+      </c>
+      <c r="N111" t="n">
+        <v>-1200</v>
+      </c>
+      <c r="O111" t="n">
+        <v>4</v>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.09 → 1.01 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23400: CE 5m +938,340 | PE 5m -1,129,635 | OTM CE +532,480 | OTM PE -413,010
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:02:13</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>23475.2</v>
+      </c>
+      <c r="F112" t="n">
+        <v>23408.5</v>
+      </c>
+      <c r="G112" t="n">
+        <v>23541.9</v>
+      </c>
+      <c r="H112" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I112" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:05:56</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>23545</v>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M112" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="N112" t="n">
+        <v>5235</v>
+      </c>
+      <c r="O112" t="n">
+        <v>4</v>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.83 → 0.84 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23400: CE 5m -546,455 | PE 5m +883,805 | OTM CE -232,375 | OTM PE +32,825
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (22.4x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:10:25</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>23569.3</v>
+      </c>
+      <c r="F113" t="n">
+        <v>23502.6</v>
+      </c>
+      <c r="G113" t="n">
+        <v>23636</v>
+      </c>
+      <c r="H113" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I113" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:14:18</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>23537.9</v>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M113" t="n">
+        <v>-31.4</v>
+      </c>
+      <c r="N113" t="n">
+        <v>-2355</v>
+      </c>
+      <c r="O113" t="n">
+        <v>4</v>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 0.79 → 0.83 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23500: CE 5m -2,399,475 | PE 5m +1,914,445 | OTM CE -950,040 | OTM PE +1,201,655
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (4.4x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:14:20</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>23539.8</v>
+      </c>
+      <c r="F114" t="n">
+        <v>23606.5</v>
+      </c>
+      <c r="G114" t="n">
+        <v>23473.1</v>
+      </c>
+      <c r="H114" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I114" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:21:11</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>23471</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="N114" t="n">
+        <v>5160</v>
+      </c>
+      <c r="O114" t="n">
+        <v>4</v>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.05 → 1.04 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23450: CE 5m +236,015 | PE 5m +494,585 | OTM CE +427,180 | OTM PE +124,410
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7681,7 +9031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O65"/>
+  <dimension ref="A1:O118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10786,6 +12136,2497 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>117</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:59:42</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>4</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>23458</v>
+      </c>
+      <c r="H66" t="n">
+        <v>23484.7</v>
+      </c>
+      <c r="I66" t="n">
+        <v>23391.3</v>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>118</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:01:33</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>4</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>23450</v>
+      </c>
+      <c r="H67" t="n">
+        <v>23476.7</v>
+      </c>
+      <c r="I67" t="n">
+        <v>23383.3</v>
+      </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>119</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:31:09</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>4</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>23534.4</v>
+      </c>
+      <c r="H68" t="n">
+        <v>23601.1</v>
+      </c>
+      <c r="I68" t="n">
+        <v>23467.7</v>
+      </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>120</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:31:31</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>4</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>23539.7</v>
+      </c>
+      <c r="H69" t="n">
+        <v>23606.4</v>
+      </c>
+      <c r="I69" t="n">
+        <v>23473</v>
+      </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>121</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:56:34</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>4</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>23561.9</v>
+      </c>
+      <c r="H70" t="n">
+        <v>23628.6</v>
+      </c>
+      <c r="I70" t="n">
+        <v>23495.2</v>
+      </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>122</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-06-03 15:07:21</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>4</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>23549.3</v>
+      </c>
+      <c r="H71" t="n">
+        <v>23616</v>
+      </c>
+      <c r="I71" t="n">
+        <v>23482.6</v>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>123</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-06-03 15:07:37</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>4</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>23551.9</v>
+      </c>
+      <c r="H72" t="n">
+        <v>23618.6</v>
+      </c>
+      <c r="I72" t="n">
+        <v>23485.2</v>
+      </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>124</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-06-03 15:07:49</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>4</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>23550.5</v>
+      </c>
+      <c r="H73" t="n">
+        <v>23617.2</v>
+      </c>
+      <c r="I73" t="n">
+        <v>23483.8</v>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>125</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-06-04 12:19:09</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>4</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>23492.2</v>
+      </c>
+      <c r="H74" t="n">
+        <v>23558.9</v>
+      </c>
+      <c r="I74" t="n">
+        <v>23425.5</v>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>126</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-06-04 12:45:08</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>4</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>23442</v>
+      </c>
+      <c r="H75" t="n">
+        <v>23508.7</v>
+      </c>
+      <c r="I75" t="n">
+        <v>23375.3</v>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>127</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-06-04 12:45:30</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>4</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>23448</v>
+      </c>
+      <c r="H76" t="n">
+        <v>23514.7</v>
+      </c>
+      <c r="I76" t="n">
+        <v>23381.3</v>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>128</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-06-04 13:36:31</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>4</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>23422</v>
+      </c>
+      <c r="H77" t="n">
+        <v>23355.3</v>
+      </c>
+      <c r="I77" t="n">
+        <v>23488.7</v>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>129</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-06-04 13:45:05</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>4</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>23419.6</v>
+      </c>
+      <c r="H78" t="n">
+        <v>23352.9</v>
+      </c>
+      <c r="I78" t="n">
+        <v>23486.3</v>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>130</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-06-04 13:46:46</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>4</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>23420</v>
+      </c>
+      <c r="H79" t="n">
+        <v>23353.3</v>
+      </c>
+      <c r="I79" t="n">
+        <v>23486.7</v>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>131</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-06-04 13:56:49</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>4</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>23409.1</v>
+      </c>
+      <c r="H80" t="n">
+        <v>23342.4</v>
+      </c>
+      <c r="I80" t="n">
+        <v>23475.8</v>
+      </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>132</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:10:12</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>4</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>23477.9</v>
+      </c>
+      <c r="H81" t="n">
+        <v>23411.2</v>
+      </c>
+      <c r="I81" t="n">
+        <v>23544.6</v>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>133</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:34:43</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>4</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>23495.1</v>
+      </c>
+      <c r="H82" t="n">
+        <v>23428.4</v>
+      </c>
+      <c r="I82" t="n">
+        <v>23561.8</v>
+      </c>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>134</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-06-04 14:58:46</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>4</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>23474</v>
+      </c>
+      <c r="H83" t="n">
+        <v>23540.7</v>
+      </c>
+      <c r="I83" t="n">
+        <v>23407.3</v>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>135</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:08:12</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>4</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>23471.7</v>
+      </c>
+      <c r="H84" t="n">
+        <v>23538.4</v>
+      </c>
+      <c r="I84" t="n">
+        <v>23405</v>
+      </c>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>136</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:08:29</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>4</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>23472.1</v>
+      </c>
+      <c r="H85" t="n">
+        <v>23538.8</v>
+      </c>
+      <c r="I85" t="n">
+        <v>23405.4</v>
+      </c>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>137</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:09:45</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>4</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>23472.5</v>
+      </c>
+      <c r="H86" t="n">
+        <v>23539.2</v>
+      </c>
+      <c r="I86" t="n">
+        <v>23405.8</v>
+      </c>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>138</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:15:50</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>4</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>23529.9</v>
+      </c>
+      <c r="H87" t="n">
+        <v>23596.6</v>
+      </c>
+      <c r="I87" t="n">
+        <v>23463.2</v>
+      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>139</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:16:43</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>4</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>23520</v>
+      </c>
+      <c r="H88" t="n">
+        <v>23586.7</v>
+      </c>
+      <c r="I88" t="n">
+        <v>23453.3</v>
+      </c>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>140</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:23:50</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>4</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>23472</v>
+      </c>
+      <c r="H89" t="n">
+        <v>23538.7</v>
+      </c>
+      <c r="I89" t="n">
+        <v>23405.3</v>
+      </c>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>141</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:26:00</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>4</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>23488.9</v>
+      </c>
+      <c r="H90" t="n">
+        <v>23555.6</v>
+      </c>
+      <c r="I90" t="n">
+        <v>23422.2</v>
+      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>142</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:32:05</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>4</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>23510</v>
+      </c>
+      <c r="H91" t="n">
+        <v>23576.7</v>
+      </c>
+      <c r="I91" t="n">
+        <v>23443.3</v>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>143</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:44:39</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>4</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>23505</v>
+      </c>
+      <c r="H92" t="n">
+        <v>23571.7</v>
+      </c>
+      <c r="I92" t="n">
+        <v>23438.3</v>
+      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>144</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:58:56</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>4</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>23469.9</v>
+      </c>
+      <c r="H93" t="n">
+        <v>23536.6</v>
+      </c>
+      <c r="I93" t="n">
+        <v>23403.2</v>
+      </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>145</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:59:16</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>4</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>23463.5</v>
+      </c>
+      <c r="H94" t="n">
+        <v>23530.2</v>
+      </c>
+      <c r="I94" t="n">
+        <v>23396.8</v>
+      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>146</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-06-05 11:59:45</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>4</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>23462</v>
+      </c>
+      <c r="H95" t="n">
+        <v>23528.7</v>
+      </c>
+      <c r="I95" t="n">
+        <v>23395.3</v>
+      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>147</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:01:30</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>23470</v>
+      </c>
+      <c r="H96" t="n">
+        <v>23536.7</v>
+      </c>
+      <c r="I96" t="n">
+        <v>23403.3</v>
+      </c>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>148</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:05:16</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>4</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>23495</v>
+      </c>
+      <c r="H97" t="n">
+        <v>23561.7</v>
+      </c>
+      <c r="I97" t="n">
+        <v>23428.3</v>
+      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>149</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:16:57</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>4</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>23499.9</v>
+      </c>
+      <c r="H98" t="n">
+        <v>23566.6</v>
+      </c>
+      <c r="I98" t="n">
+        <v>23433.2</v>
+      </c>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>150</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:17:15</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>4</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
+        <v>23499</v>
+      </c>
+      <c r="H99" t="n">
+        <v>23565.7</v>
+      </c>
+      <c r="I99" t="n">
+        <v>23432.3</v>
+      </c>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>151</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:34:44</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>4</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>23480</v>
+      </c>
+      <c r="H100" t="n">
+        <v>23546.7</v>
+      </c>
+      <c r="I100" t="n">
+        <v>23413.3</v>
+      </c>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>152</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:36:02</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>4</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>23488.8</v>
+      </c>
+      <c r="H101" t="n">
+        <v>23555.5</v>
+      </c>
+      <c r="I101" t="n">
+        <v>23422.1</v>
+      </c>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>153</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:37:42</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>4</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
+        <v>23457</v>
+      </c>
+      <c r="H102" t="n">
+        <v>23523.7</v>
+      </c>
+      <c r="I102" t="n">
+        <v>23390.3</v>
+      </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>154</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:39:19</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
+        <v>23460</v>
+      </c>
+      <c r="H103" t="n">
+        <v>23526.7</v>
+      </c>
+      <c r="I103" t="n">
+        <v>23393.3</v>
+      </c>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>155</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:39:59</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>4</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G104" t="n">
+        <v>23472</v>
+      </c>
+      <c r="H104" t="n">
+        <v>23538.7</v>
+      </c>
+      <c r="I104" t="n">
+        <v>23405.3</v>
+      </c>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>156</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:42:48</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>4</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
+        <v>23460</v>
+      </c>
+      <c r="H105" t="n">
+        <v>23526.7</v>
+      </c>
+      <c r="I105" t="n">
+        <v>23393.3</v>
+      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>157</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:44:59</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>4</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>23445</v>
+      </c>
+      <c r="H106" t="n">
+        <v>23511.7</v>
+      </c>
+      <c r="I106" t="n">
+        <v>23378.3</v>
+      </c>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>158</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:45:34</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G107" t="n">
+        <v>23438</v>
+      </c>
+      <c r="H107" t="n">
+        <v>23504.7</v>
+      </c>
+      <c r="I107" t="n">
+        <v>23371.3</v>
+      </c>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>159</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:45:53</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>4</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>23445</v>
+      </c>
+      <c r="H108" t="n">
+        <v>23511.7</v>
+      </c>
+      <c r="I108" t="n">
+        <v>23378.3</v>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>160</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:13:58</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>4</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G109" t="n">
+        <v>23420.8</v>
+      </c>
+      <c r="H109" t="n">
+        <v>23487.5</v>
+      </c>
+      <c r="I109" t="n">
+        <v>23354.1</v>
+      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>161</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:14:32</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>4</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>23412</v>
+      </c>
+      <c r="H110" t="n">
+        <v>23478.7</v>
+      </c>
+      <c r="I110" t="n">
+        <v>23345.3</v>
+      </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>162</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:15:00</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>4</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>23410</v>
+      </c>
+      <c r="H111" t="n">
+        <v>23476.7</v>
+      </c>
+      <c r="I111" t="n">
+        <v>23343.3</v>
+      </c>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>163</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:16:06</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>4</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>23425</v>
+      </c>
+      <c r="H112" t="n">
+        <v>23491.7</v>
+      </c>
+      <c r="I112" t="n">
+        <v>23358.3</v>
+      </c>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>164</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:18:09</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>4</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>23431.7</v>
+      </c>
+      <c r="H113" t="n">
+        <v>23498.4</v>
+      </c>
+      <c r="I113" t="n">
+        <v>23365</v>
+      </c>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>165</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:39:27</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>4</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G114" t="n">
+        <v>23388</v>
+      </c>
+      <c r="H114" t="n">
+        <v>23454.7</v>
+      </c>
+      <c r="I114" t="n">
+        <v>23321.3</v>
+      </c>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>166</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:41:09</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>4</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G115" t="n">
+        <v>23390</v>
+      </c>
+      <c r="H115" t="n">
+        <v>23456.7</v>
+      </c>
+      <c r="I115" t="n">
+        <v>23323.3</v>
+      </c>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>167</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-06-05 13:59:51</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>4</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G116" t="n">
+        <v>23390</v>
+      </c>
+      <c r="H116" t="n">
+        <v>23456.7</v>
+      </c>
+      <c r="I116" t="n">
+        <v>23323.3</v>
+      </c>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>168</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-06-05 14:25:36</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>4</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>23400</v>
+      </c>
+      <c r="H117" t="n">
+        <v>23466.7</v>
+      </c>
+      <c r="I117" t="n">
+        <v>23333.3</v>
+      </c>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>169</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-06-05 14:34:47</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>4</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>23421</v>
+      </c>
+      <c r="H118" t="n">
+        <v>23354.3</v>
+      </c>
+      <c r="I118" t="n">
+        <v>23487.7</v>
+      </c>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10823,7 +14664,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3">
@@ -10833,7 +14674,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -10843,7 +14684,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5">
@@ -10854,7 +14695,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35.79%</t>
+          <t>38.05%</t>
         </is>
       </c>
     </row>
@@ -10866,7 +14707,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 2,392.50</t>
+          <t>Rs. 9,562.50</t>
         </is>
       </c>
     </row>
@@ -10878,7 +14719,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>31.90</t>
+          <t>127.50</t>
         </is>
       </c>
     </row>
@@ -10890,7 +14731,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs. 3,950.74</t>
+          <t>Rs. 3,896.51</t>
         </is>
       </c>
     </row>
@@ -10902,7 +14743,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -2,162.83</t>
+          <t>Rs. -2,256.96</t>
         </is>
       </c>
     </row>
@@ -10938,7 +14779,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>1.06</t>
         </is>
       </c>
     </row>
@@ -10949,7 +14790,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>64</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14">
@@ -10960,7 +14801,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-01 14:08:32</t>
+          <t>2026-06-05 14:53:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 06-06-2026 22:35:53.13
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q114"/>
+  <dimension ref="A1:Q113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -435,8 +435,8 @@
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
@@ -7147,31 +7147,31 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-05-29 15:04:06</t>
+          <t>2026-06-01 10:57:03</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>NSE:NIFTY26MAYFUT</t>
+          <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>23727.4</v>
+        <v>23661.5</v>
       </c>
       <c r="F90" t="n">
-        <v>23754.1</v>
+        <v>23634.8</v>
       </c>
       <c r="G90" t="n">
-        <v>23660.7</v>
+        <v>23728.2</v>
       </c>
       <c r="H90" t="n">
         <v>26.7</v>
@@ -7181,11 +7181,11 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>2026-05-29 15:04:07</t>
+          <t>2026-06-01 11:29:52</t>
         </is>
       </c>
       <c r="K90" t="n">
-        <v>23913</v>
+        <v>23632</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -7193,95 +7193,20 @@
         </is>
       </c>
       <c r="M90" t="n">
-        <v>-185.6</v>
+        <v>-29.5</v>
       </c>
       <c r="N90" t="n">
-        <v>-13920</v>
+        <v>-2212.5</v>
       </c>
       <c r="O90" t="n">
         <v>4</v>
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>BEARISH</t>
+          <t>BULLISH</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
-──────────────────────────────
-🎯 INSTITUTIONAL CHECKLIST (4/4)
-  ✅ 1. PCR Trend: PCR Falling 0.97 → 0.95 (Bearish momentum)
-  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23600: CE 5m +810,485 | PE 5m -225,875 | OTM CE +632,515 | OTM PE +427,570
-  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
-  ✅ 4. Order Flow: Sell dominant (0.0x)
-  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
-──────────────────────────────</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>2026-06-01 10:57:03</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>NSE:NIFTY26JUNFUT</t>
-        </is>
-      </c>
-      <c r="E91" t="n">
-        <v>23661.5</v>
-      </c>
-      <c r="F91" t="n">
-        <v>23634.8</v>
-      </c>
-      <c r="G91" t="n">
-        <v>23728.2</v>
-      </c>
-      <c r="H91" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="I91" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>2026-06-01 11:29:52</t>
-        </is>
-      </c>
-      <c r="K91" t="n">
-        <v>23632</v>
-      </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>SL_HIT</t>
-        </is>
-      </c>
-      <c r="M91" t="n">
-        <v>-29.5</v>
-      </c>
-      <c r="N91" t="n">
-        <v>-2212.5</v>
-      </c>
-      <c r="O91" t="n">
-        <v>4</v>
-      </c>
-      <c r="P91" t="inlineStr">
-        <is>
-          <t>BULLISH</t>
-        </is>
-      </c>
-      <c r="Q91" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7295,68 +7220,68 @@
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="n">
+    <row r="91">
+      <c r="A91" t="n">
         <v>91</v>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>2026-06-01 11:36:17</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E92" t="n">
+      <c r="E91" t="n">
         <v>23624.9</v>
       </c>
-      <c r="F92" t="n">
+      <c r="F91" t="n">
         <v>23651.6</v>
       </c>
-      <c r="G92" t="n">
+      <c r="G91" t="n">
         <v>23558.2</v>
       </c>
-      <c r="H92" t="n">
+      <c r="H91" t="n">
         <v>26.7</v>
       </c>
-      <c r="I92" t="n">
+      <c r="I91" t="n">
         <v>66.7</v>
       </c>
-      <c r="J92" t="inlineStr">
+      <c r="J91" t="inlineStr">
         <is>
           <t>2026-06-01 11:59:27</t>
         </is>
       </c>
-      <c r="K92" t="n">
+      <c r="K91" t="n">
         <v>23558</v>
       </c>
-      <c r="L92" t="inlineStr">
+      <c r="L91" t="inlineStr">
         <is>
           <t>TARGET_HIT</t>
         </is>
       </c>
-      <c r="M92" t="n">
+      <c r="M91" t="n">
         <v>66.90000000000001</v>
       </c>
-      <c r="N92" t="n">
+      <c r="N91" t="n">
         <v>5017.5</v>
       </c>
-      <c r="O92" t="n">
-        <v>4</v>
-      </c>
-      <c r="P92" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q92" t="inlineStr">
+      <c r="O91" t="n">
+        <v>4</v>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7370,68 +7295,68 @@
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" t="n">
+    <row r="92">
+      <c r="A92" t="n">
         <v>92</v>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>2026-06-01 12:03:47</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E93" t="n">
+      <c r="E92" t="n">
         <v>23560</v>
       </c>
-      <c r="F93" t="n">
+      <c r="F92" t="n">
         <v>23586.7</v>
       </c>
-      <c r="G93" t="n">
+      <c r="G92" t="n">
         <v>23493.3</v>
       </c>
-      <c r="H93" t="n">
+      <c r="H92" t="n">
         <v>26.7</v>
       </c>
-      <c r="I93" t="n">
+      <c r="I92" t="n">
         <v>66.7</v>
       </c>
-      <c r="J93" t="inlineStr">
+      <c r="J92" t="inlineStr">
         <is>
           <t>2026-06-01 12:14:22</t>
         </is>
       </c>
-      <c r="K93" t="n">
+      <c r="K92" t="n">
         <v>23587.7</v>
       </c>
-      <c r="L93" t="inlineStr">
+      <c r="L92" t="inlineStr">
         <is>
           <t>SL_HIT</t>
         </is>
       </c>
-      <c r="M93" t="n">
+      <c r="M92" t="n">
         <v>-27.7</v>
       </c>
-      <c r="N93" t="n">
+      <c r="N92" t="n">
         <v>-2077.5</v>
       </c>
-      <c r="O93" t="n">
-        <v>4</v>
-      </c>
-      <c r="P93" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q93" t="inlineStr">
+      <c r="O92" t="n">
+        <v>4</v>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7445,68 +7370,68 @@
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="n">
+    <row r="93">
+      <c r="A93" t="n">
         <v>93</v>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>2026-06-01 12:17:34</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E94" t="n">
+      <c r="E93" t="n">
         <v>23578.5</v>
       </c>
-      <c r="F94" t="n">
+      <c r="F93" t="n">
         <v>23551.8</v>
       </c>
-      <c r="G94" t="n">
+      <c r="G93" t="n">
         <v>23645.2</v>
       </c>
-      <c r="H94" t="n">
+      <c r="H93" t="n">
         <v>26.7</v>
       </c>
-      <c r="I94" t="n">
+      <c r="I93" t="n">
         <v>66.7</v>
       </c>
-      <c r="J94" t="inlineStr">
+      <c r="J93" t="inlineStr">
         <is>
           <t>2026-06-01 12:34:30</t>
         </is>
       </c>
-      <c r="K94" t="n">
+      <c r="K93" t="n">
         <v>23570</v>
       </c>
-      <c r="L94" t="inlineStr">
+      <c r="L93" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M94" t="n">
+      <c r="M93" t="n">
         <v>-8.5</v>
       </c>
-      <c r="N94" t="n">
+      <c r="N93" t="n">
         <v>-637.5</v>
       </c>
-      <c r="O94" t="n">
-        <v>4</v>
-      </c>
-      <c r="P94" t="inlineStr">
+      <c r="O93" t="n">
+        <v>4</v>
+      </c>
+      <c r="P93" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q94" t="inlineStr">
+      <c r="Q93" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7520,68 +7445,68 @@
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" t="n">
+    <row r="94">
+      <c r="A94" t="n">
         <v>94</v>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>2026-06-01 12:34:32</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E95" t="n">
+      <c r="E94" t="n">
         <v>23571</v>
       </c>
-      <c r="F95" t="n">
+      <c r="F94" t="n">
         <v>23597.7</v>
       </c>
-      <c r="G95" t="n">
+      <c r="G94" t="n">
         <v>23504.3</v>
       </c>
-      <c r="H95" t="n">
+      <c r="H94" t="n">
         <v>26.7</v>
       </c>
-      <c r="I95" t="n">
+      <c r="I94" t="n">
         <v>66.7</v>
       </c>
-      <c r="J95" t="inlineStr">
+      <c r="J94" t="inlineStr">
         <is>
           <t>2026-06-01 12:43:05</t>
         </is>
       </c>
-      <c r="K95" t="n">
+      <c r="K94" t="n">
         <v>23570.5</v>
       </c>
-      <c r="L95" t="inlineStr">
+      <c r="L94" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M95" t="n">
+      <c r="M94" t="n">
         <v>0.5</v>
       </c>
-      <c r="N95" t="n">
+      <c r="N94" t="n">
         <v>37.5</v>
       </c>
-      <c r="O95" t="n">
-        <v>4</v>
-      </c>
-      <c r="P95" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q95" t="inlineStr">
+      <c r="O94" t="n">
+        <v>4</v>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7595,68 +7520,68 @@
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="n">
+    <row r="95">
+      <c r="A95" t="n">
         <v>95</v>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>2026-06-01 12:43:06</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E96" t="n">
+      <c r="E95" t="n">
         <v>23570.5</v>
       </c>
-      <c r="F96" t="n">
+      <c r="F95" t="n">
         <v>23543.8</v>
       </c>
-      <c r="G96" t="n">
+      <c r="G95" t="n">
         <v>23637.2</v>
       </c>
-      <c r="H96" t="n">
+      <c r="H95" t="n">
         <v>26.7</v>
       </c>
-      <c r="I96" t="n">
+      <c r="I95" t="n">
         <v>66.7</v>
       </c>
-      <c r="J96" t="inlineStr">
+      <c r="J95" t="inlineStr">
         <is>
           <t>2026-06-01 13:08:10</t>
         </is>
       </c>
-      <c r="K96" t="n">
+      <c r="K95" t="n">
         <v>23543.5</v>
       </c>
-      <c r="L96" t="inlineStr">
+      <c r="L95" t="inlineStr">
         <is>
           <t>SL_HIT</t>
         </is>
       </c>
-      <c r="M96" t="n">
+      <c r="M95" t="n">
         <v>-27</v>
       </c>
-      <c r="N96" t="n">
+      <c r="N95" t="n">
         <v>-2025</v>
       </c>
-      <c r="O96" t="n">
-        <v>4</v>
-      </c>
-      <c r="P96" t="inlineStr">
+      <c r="O95" t="n">
+        <v>4</v>
+      </c>
+      <c r="P95" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q96" t="inlineStr">
+      <c r="Q95" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7670,68 +7595,68 @@
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" t="n">
+    <row r="96">
+      <c r="A96" t="n">
         <v>96</v>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>2026-06-03 09:47:46</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E97" t="n">
+      <c r="E96" t="n">
         <v>23334</v>
       </c>
-      <c r="F97" t="n">
+      <c r="F96" t="n">
         <v>23400.7</v>
       </c>
-      <c r="G97" t="n">
+      <c r="G96" t="n">
         <v>23267.3</v>
       </c>
-      <c r="H97" t="n">
+      <c r="H96" t="n">
         <v>66.7</v>
       </c>
-      <c r="I97" t="n">
+      <c r="I96" t="n">
         <v>66.7</v>
       </c>
-      <c r="J97" t="inlineStr">
+      <c r="J96" t="inlineStr">
         <is>
           <t>2026-06-03 11:09:15</t>
         </is>
       </c>
-      <c r="K97" t="n">
+      <c r="K96" t="n">
         <v>23264.5</v>
       </c>
-      <c r="L97" t="inlineStr">
+      <c r="L96" t="inlineStr">
         <is>
           <t>TARGET_HIT</t>
         </is>
       </c>
-      <c r="M97" t="n">
+      <c r="M96" t="n">
         <v>69.5</v>
       </c>
-      <c r="N97" t="n">
+      <c r="N96" t="n">
         <v>5212.5</v>
       </c>
-      <c r="O97" t="n">
-        <v>4</v>
-      </c>
-      <c r="P97" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q97" t="inlineStr">
+      <c r="O96" t="n">
+        <v>4</v>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7745,68 +7670,68 @@
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" t="n">
+    <row r="97">
+      <c r="A97" t="n">
         <v>97</v>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>2026-06-03 11:09:46</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E98" t="n">
+      <c r="E97" t="n">
         <v>23262</v>
       </c>
-      <c r="F98" t="n">
+      <c r="F97" t="n">
         <v>23328.7</v>
       </c>
-      <c r="G98" t="n">
+      <c r="G97" t="n">
         <v>23195.3</v>
       </c>
-      <c r="H98" t="n">
+      <c r="H97" t="n">
         <v>66.7</v>
       </c>
-      <c r="I98" t="n">
+      <c r="I97" t="n">
         <v>66.7</v>
       </c>
-      <c r="J98" t="inlineStr">
+      <c r="J97" t="inlineStr">
         <is>
           <t>2026-06-03 12:30:40</t>
         </is>
       </c>
-      <c r="K98" t="n">
+      <c r="K97" t="n">
         <v>23330</v>
       </c>
-      <c r="L98" t="inlineStr">
+      <c r="L97" t="inlineStr">
         <is>
           <t>SL_HIT</t>
         </is>
       </c>
-      <c r="M98" t="n">
+      <c r="M97" t="n">
         <v>-68</v>
       </c>
-      <c r="N98" t="n">
+      <c r="N97" t="n">
         <v>-5100</v>
       </c>
-      <c r="O98" t="n">
-        <v>4</v>
-      </c>
-      <c r="P98" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q98" t="inlineStr">
+      <c r="O97" t="n">
+        <v>4</v>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7820,68 +7745,68 @@
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" t="n">
+    <row r="98">
+      <c r="A98" t="n">
         <v>98</v>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>2026-06-03 12:35:25</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D98" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E99" t="n">
+      <c r="E98" t="n">
         <v>23370</v>
       </c>
-      <c r="F99" t="n">
+      <c r="F98" t="n">
         <v>23303.3</v>
       </c>
-      <c r="G99" t="n">
+      <c r="G98" t="n">
         <v>23436.7</v>
       </c>
-      <c r="H99" t="n">
+      <c r="H98" t="n">
         <v>66.7</v>
       </c>
-      <c r="I99" t="n">
+      <c r="I98" t="n">
         <v>66.7</v>
       </c>
-      <c r="J99" t="inlineStr">
+      <c r="J98" t="inlineStr">
         <is>
           <t>2026-06-03 12:53:51</t>
         </is>
       </c>
-      <c r="K99" t="n">
+      <c r="K98" t="n">
         <v>23375.1</v>
       </c>
-      <c r="L99" t="inlineStr">
+      <c r="L98" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M99" t="n">
+      <c r="M98" t="n">
         <v>5.1</v>
       </c>
-      <c r="N99" t="n">
+      <c r="N98" t="n">
         <v>382.5</v>
       </c>
-      <c r="O99" t="n">
-        <v>4</v>
-      </c>
-      <c r="P99" t="inlineStr">
+      <c r="O98" t="n">
+        <v>4</v>
+      </c>
+      <c r="P98" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q99" t="inlineStr">
+      <c r="Q98" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7895,68 +7820,68 @@
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" t="n">
+    <row r="99">
+      <c r="A99" t="n">
         <v>99</v>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>2026-06-03 12:53:51</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E100" t="n">
+      <c r="E99" t="n">
         <v>23375.1</v>
       </c>
-      <c r="F100" t="n">
+      <c r="F99" t="n">
         <v>23441.8</v>
       </c>
-      <c r="G100" t="n">
+      <c r="G99" t="n">
         <v>23308.4</v>
       </c>
-      <c r="H100" t="n">
+      <c r="H99" t="n">
         <v>66.7</v>
       </c>
-      <c r="I100" t="n">
+      <c r="I99" t="n">
         <v>66.7</v>
       </c>
-      <c r="J100" t="inlineStr">
+      <c r="J99" t="inlineStr">
         <is>
           <t>2026-06-03 13:15:38</t>
         </is>
       </c>
-      <c r="K100" t="n">
+      <c r="K99" t="n">
         <v>23392</v>
       </c>
-      <c r="L100" t="inlineStr">
+      <c r="L99" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M100" t="n">
+      <c r="M99" t="n">
         <v>-16.9</v>
       </c>
-      <c r="N100" t="n">
+      <c r="N99" t="n">
         <v>-1267.5</v>
       </c>
-      <c r="O100" t="n">
-        <v>4</v>
-      </c>
-      <c r="P100" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q100" t="inlineStr">
+      <c r="O99" t="n">
+        <v>4</v>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -7970,68 +7895,68 @@
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" t="n">
+    <row r="100">
+      <c r="A100" t="n">
         <v>100</v>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>2026-06-03 13:15:39</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D100" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E101" t="n">
+      <c r="E100" t="n">
         <v>23389.3</v>
       </c>
-      <c r="F101" t="n">
+      <c r="F100" t="n">
         <v>23322.6</v>
       </c>
-      <c r="G101" t="n">
+      <c r="G100" t="n">
         <v>23456</v>
       </c>
-      <c r="H101" t="n">
+      <c r="H100" t="n">
         <v>66.7</v>
       </c>
-      <c r="I101" t="n">
+      <c r="I100" t="n">
         <v>66.7</v>
       </c>
-      <c r="J101" t="inlineStr">
+      <c r="J100" t="inlineStr">
         <is>
           <t>2026-06-03 13:46:56</t>
         </is>
       </c>
-      <c r="K101" t="n">
+      <c r="K100" t="n">
         <v>23456.5</v>
       </c>
-      <c r="L101" t="inlineStr">
+      <c r="L100" t="inlineStr">
         <is>
           <t>TARGET_HIT</t>
         </is>
       </c>
-      <c r="M101" t="n">
+      <c r="M100" t="n">
         <v>67.2</v>
       </c>
-      <c r="N101" t="n">
+      <c r="N100" t="n">
         <v>5040</v>
       </c>
-      <c r="O101" t="n">
-        <v>4</v>
-      </c>
-      <c r="P101" t="inlineStr">
+      <c r="O100" t="n">
+        <v>4</v>
+      </c>
+      <c r="P100" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q101" t="inlineStr">
+      <c r="Q100" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8045,68 +7970,68 @@
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" t="n">
+    <row r="101">
+      <c r="A101" t="n">
         <v>101</v>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>2026-06-03 14:02:50</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E102" t="n">
+      <c r="E101" t="n">
         <v>23480.8</v>
       </c>
-      <c r="F102" t="n">
+      <c r="F101" t="n">
         <v>23547.5</v>
       </c>
-      <c r="G102" t="n">
+      <c r="G101" t="n">
         <v>23414.1</v>
       </c>
-      <c r="H102" t="n">
+      <c r="H101" t="n">
         <v>66.7</v>
       </c>
-      <c r="I102" t="n">
+      <c r="I101" t="n">
         <v>66.7</v>
       </c>
-      <c r="J102" t="inlineStr">
+      <c r="J101" t="inlineStr">
         <is>
           <t>2026-06-03 14:23:04</t>
         </is>
       </c>
-      <c r="K102" t="n">
+      <c r="K101" t="n">
         <v>23549</v>
       </c>
-      <c r="L102" t="inlineStr">
+      <c r="L101" t="inlineStr">
         <is>
           <t>SL_HIT</t>
         </is>
       </c>
-      <c r="M102" t="n">
+      <c r="M101" t="n">
         <v>-68.2</v>
       </c>
-      <c r="N102" t="n">
+      <c r="N101" t="n">
         <v>-5115</v>
       </c>
-      <c r="O102" t="n">
-        <v>4</v>
-      </c>
-      <c r="P102" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q102" t="inlineStr">
+      <c r="O101" t="n">
+        <v>4</v>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8120,68 +8045,68 @@
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" t="n">
+    <row r="102">
+      <c r="A102" t="n">
         <v>102</v>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>2026-06-04 09:33:54</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E103" t="n">
+      <c r="E102" t="n">
         <v>23405.9</v>
       </c>
-      <c r="F103" t="n">
+      <c r="F102" t="n">
         <v>23472.6</v>
       </c>
-      <c r="G103" t="n">
+      <c r="G102" t="n">
         <v>23339.2</v>
       </c>
-      <c r="H103" t="n">
+      <c r="H102" t="n">
         <v>66.7</v>
       </c>
-      <c r="I103" t="n">
+      <c r="I102" t="n">
         <v>66.7</v>
       </c>
-      <c r="J103" t="inlineStr">
+      <c r="J102" t="inlineStr">
         <is>
           <t>2026-06-04 09:41:05</t>
         </is>
       </c>
-      <c r="K103" t="n">
+      <c r="K102" t="n">
         <v>23380.1</v>
       </c>
-      <c r="L103" t="inlineStr">
+      <c r="L102" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M103" t="n">
+      <c r="M102" t="n">
         <v>25.8</v>
       </c>
-      <c r="N103" t="n">
+      <c r="N102" t="n">
         <v>1935</v>
       </c>
-      <c r="O103" t="n">
-        <v>4</v>
-      </c>
-      <c r="P103" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q103" t="inlineStr">
+      <c r="O102" t="n">
+        <v>4</v>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8195,68 +8120,68 @@
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="n">
+    <row r="103">
+      <c r="A103" t="n">
         <v>103</v>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>2026-06-04 09:41:05</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
+      <c r="D103" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E104" t="n">
+      <c r="E103" t="n">
         <v>23381.3</v>
       </c>
-      <c r="F104" t="n">
+      <c r="F103" t="n">
         <v>23314.6</v>
       </c>
-      <c r="G104" t="n">
+      <c r="G103" t="n">
         <v>23448</v>
       </c>
-      <c r="H104" t="n">
+      <c r="H103" t="n">
         <v>66.7</v>
       </c>
-      <c r="I104" t="n">
+      <c r="I103" t="n">
         <v>66.7</v>
       </c>
-      <c r="J104" t="inlineStr">
+      <c r="J103" t="inlineStr">
         <is>
           <t>2026-06-04 09:49:03</t>
         </is>
       </c>
-      <c r="K104" t="n">
+      <c r="K103" t="n">
         <v>23449</v>
       </c>
-      <c r="L104" t="inlineStr">
+      <c r="L103" t="inlineStr">
         <is>
           <t>TARGET_HIT</t>
         </is>
       </c>
-      <c r="M104" t="n">
+      <c r="M103" t="n">
         <v>67.7</v>
       </c>
-      <c r="N104" t="n">
+      <c r="N103" t="n">
         <v>5077.5</v>
       </c>
-      <c r="O104" t="n">
-        <v>4</v>
-      </c>
-      <c r="P104" t="inlineStr">
+      <c r="O103" t="n">
+        <v>4</v>
+      </c>
+      <c r="P103" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q104" t="inlineStr">
+      <c r="Q103" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8270,68 +8195,68 @@
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" t="n">
+    <row r="104">
+      <c r="A104" t="n">
         <v>104</v>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B104" t="inlineStr">
         <is>
           <t>2026-06-04 10:30:20</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D104" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E105" t="n">
+      <c r="E104" t="n">
         <v>23490</v>
       </c>
-      <c r="F105" t="n">
+      <c r="F104" t="n">
         <v>23423.3</v>
       </c>
-      <c r="G105" t="n">
+      <c r="G104" t="n">
         <v>23556.7</v>
       </c>
-      <c r="H105" t="n">
+      <c r="H104" t="n">
         <v>66.7</v>
       </c>
-      <c r="I105" t="n">
+      <c r="I104" t="n">
         <v>66.7</v>
       </c>
-      <c r="J105" t="inlineStr">
+      <c r="J104" t="inlineStr">
         <is>
           <t>2026-06-04 10:33:40</t>
         </is>
       </c>
-      <c r="K105" t="n">
+      <c r="K104" t="n">
         <v>23460</v>
       </c>
-      <c r="L105" t="inlineStr">
+      <c r="L104" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M105" t="n">
+      <c r="M104" t="n">
         <v>-30</v>
       </c>
-      <c r="N105" t="n">
+      <c r="N104" t="n">
         <v>-2250</v>
       </c>
-      <c r="O105" t="n">
-        <v>4</v>
-      </c>
-      <c r="P105" t="inlineStr">
+      <c r="O104" t="n">
+        <v>4</v>
+      </c>
+      <c r="P104" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q105" t="inlineStr">
+      <c r="Q104" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8345,68 +8270,68 @@
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" t="n">
+    <row r="105">
+      <c r="A105" t="n">
         <v>105</v>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B105" t="inlineStr">
         <is>
           <t>2026-06-04 10:33:41</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E106" t="n">
+      <c r="E105" t="n">
         <v>23462.6</v>
       </c>
-      <c r="F106" t="n">
+      <c r="F105" t="n">
         <v>23529.3</v>
       </c>
-      <c r="G106" t="n">
+      <c r="G105" t="n">
         <v>23395.9</v>
       </c>
-      <c r="H106" t="n">
+      <c r="H105" t="n">
         <v>66.7</v>
       </c>
-      <c r="I106" t="n">
+      <c r="I105" t="n">
         <v>66.7</v>
       </c>
-      <c r="J106" t="inlineStr">
+      <c r="J105" t="inlineStr">
         <is>
           <t>2026-06-04 10:51:08</t>
         </is>
       </c>
-      <c r="K106" t="n">
+      <c r="K105" t="n">
         <v>23481</v>
       </c>
-      <c r="L106" t="inlineStr">
+      <c r="L105" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M106" t="n">
+      <c r="M105" t="n">
         <v>-18.4</v>
       </c>
-      <c r="N106" t="n">
+      <c r="N105" t="n">
         <v>-1380</v>
       </c>
-      <c r="O106" t="n">
-        <v>4</v>
-      </c>
-      <c r="P106" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q106" t="inlineStr">
+      <c r="O105" t="n">
+        <v>4</v>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8420,68 +8345,68 @@
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="n">
+    <row r="106">
+      <c r="A106" t="n">
         <v>106</v>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t>2026-06-04 10:51:09</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr">
+      <c r="D106" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E107" t="n">
+      <c r="E106" t="n">
         <v>23481</v>
       </c>
-      <c r="F107" t="n">
+      <c r="F106" t="n">
         <v>23414.3</v>
       </c>
-      <c r="G107" t="n">
+      <c r="G106" t="n">
         <v>23547.7</v>
       </c>
-      <c r="H107" t="n">
+      <c r="H106" t="n">
         <v>66.7</v>
       </c>
-      <c r="I107" t="n">
+      <c r="I106" t="n">
         <v>66.7</v>
       </c>
-      <c r="J107" t="inlineStr">
+      <c r="J106" t="inlineStr">
         <is>
           <t>2026-06-04 11:32:16</t>
         </is>
       </c>
-      <c r="K107" t="n">
+      <c r="K106" t="n">
         <v>23413.2</v>
       </c>
-      <c r="L107" t="inlineStr">
+      <c r="L106" t="inlineStr">
         <is>
           <t>SL_HIT</t>
         </is>
       </c>
-      <c r="M107" t="n">
+      <c r="M106" t="n">
         <v>-67.8</v>
       </c>
-      <c r="N107" t="n">
+      <c r="N106" t="n">
         <v>-5085</v>
       </c>
-      <c r="O107" t="n">
-        <v>4</v>
-      </c>
-      <c r="P107" t="inlineStr">
+      <c r="O106" t="n">
+        <v>4</v>
+      </c>
+      <c r="P106" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q107" t="inlineStr">
+      <c r="Q106" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8495,68 +8420,68 @@
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" t="n">
+    <row r="107">
+      <c r="A107" t="n">
         <v>107</v>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t>2026-06-05 09:54:05</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E108" t="n">
+      <c r="E107" t="n">
         <v>23538.3</v>
       </c>
-      <c r="F108" t="n">
+      <c r="F107" t="n">
         <v>23605</v>
       </c>
-      <c r="G108" t="n">
+      <c r="G107" t="n">
         <v>23471.6</v>
       </c>
-      <c r="H108" t="n">
+      <c r="H107" t="n">
         <v>66.7</v>
       </c>
-      <c r="I108" t="n">
+      <c r="I107" t="n">
         <v>66.7</v>
       </c>
-      <c r="J108" t="inlineStr">
+      <c r="J107" t="inlineStr">
         <is>
           <t>2026-06-05 10:10:37</t>
         </is>
       </c>
-      <c r="K108" t="n">
+      <c r="K107" t="n">
         <v>23569</v>
       </c>
-      <c r="L108" t="inlineStr">
+      <c r="L107" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M108" t="n">
+      <c r="M107" t="n">
         <v>-30.7</v>
       </c>
-      <c r="N108" t="n">
+      <c r="N107" t="n">
         <v>-2302.5</v>
       </c>
-      <c r="O108" t="n">
-        <v>4</v>
-      </c>
-      <c r="P108" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q108" t="inlineStr">
+      <c r="O107" t="n">
+        <v>4</v>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8570,68 +8495,68 @@
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" t="n">
+    <row r="108">
+      <c r="A108" t="n">
         <v>108</v>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B108" t="inlineStr">
         <is>
           <t>2026-06-05 10:10:38</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C108" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D108" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E109" t="n">
+      <c r="E108" t="n">
         <v>23559.9</v>
       </c>
-      <c r="F109" t="n">
+      <c r="F108" t="n">
         <v>23493.2</v>
       </c>
-      <c r="G109" t="n">
+      <c r="G108" t="n">
         <v>23626.6</v>
       </c>
-      <c r="H109" t="n">
+      <c r="H108" t="n">
         <v>66.7</v>
       </c>
-      <c r="I109" t="n">
+      <c r="I108" t="n">
         <v>66.7</v>
       </c>
-      <c r="J109" t="inlineStr">
+      <c r="J108" t="inlineStr">
         <is>
           <t>2026-06-05 10:17:53</t>
         </is>
       </c>
-      <c r="K109" t="n">
+      <c r="K108" t="n">
         <v>23560</v>
       </c>
-      <c r="L109" t="inlineStr">
+      <c r="L108" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M109" t="n">
+      <c r="M108" t="n">
         <v>0.1</v>
       </c>
-      <c r="N109" t="n">
+      <c r="N108" t="n">
         <v>7.5</v>
       </c>
-      <c r="O109" t="n">
-        <v>4</v>
-      </c>
-      <c r="P109" t="inlineStr">
+      <c r="O108" t="n">
+        <v>4</v>
+      </c>
+      <c r="P108" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q109" t="inlineStr">
+      <c r="Q108" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8645,68 +8570,68 @@
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" t="n">
+    <row r="109">
+      <c r="A109" t="n">
         <v>109</v>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B109" t="inlineStr">
         <is>
           <t>2026-06-05 10:17:54</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E110" t="n">
+      <c r="E109" t="n">
         <v>23545</v>
       </c>
-      <c r="F110" t="n">
+      <c r="F109" t="n">
         <v>23611.7</v>
       </c>
-      <c r="G110" t="n">
+      <c r="G109" t="n">
         <v>23478.3</v>
       </c>
-      <c r="H110" t="n">
+      <c r="H109" t="n">
         <v>66.7</v>
       </c>
-      <c r="I110" t="n">
+      <c r="I109" t="n">
         <v>66.7</v>
       </c>
-      <c r="J110" t="inlineStr">
+      <c r="J109" t="inlineStr">
         <is>
           <t>2026-06-05 10:36:10</t>
         </is>
       </c>
-      <c r="K110" t="n">
+      <c r="K109" t="n">
         <v>23476</v>
       </c>
-      <c r="L110" t="inlineStr">
+      <c r="L109" t="inlineStr">
         <is>
           <t>TARGET_HIT</t>
         </is>
       </c>
-      <c r="M110" t="n">
+      <c r="M109" t="n">
         <v>69</v>
       </c>
-      <c r="N110" t="n">
+      <c r="N109" t="n">
         <v>5175</v>
       </c>
-      <c r="O110" t="n">
-        <v>4</v>
-      </c>
-      <c r="P110" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q110" t="inlineStr">
+      <c r="O109" t="n">
+        <v>4</v>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8720,68 +8645,68 @@
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" t="n">
+    <row r="110">
+      <c r="A110" t="n">
         <v>110</v>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B110" t="inlineStr">
         <is>
           <t>2026-06-05 10:38:26</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E111" t="n">
+      <c r="E110" t="n">
         <v>23464</v>
       </c>
-      <c r="F111" t="n">
+      <c r="F110" t="n">
         <v>23530.7</v>
       </c>
-      <c r="G111" t="n">
+      <c r="G110" t="n">
         <v>23397.3</v>
       </c>
-      <c r="H111" t="n">
+      <c r="H110" t="n">
         <v>66.7</v>
       </c>
-      <c r="I111" t="n">
+      <c r="I110" t="n">
         <v>66.7</v>
       </c>
-      <c r="J111" t="inlineStr">
+      <c r="J110" t="inlineStr">
         <is>
           <t>2026-06-05 11:02:12</t>
         </is>
       </c>
-      <c r="K111" t="n">
+      <c r="K110" t="n">
         <v>23480</v>
       </c>
-      <c r="L111" t="inlineStr">
+      <c r="L110" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M111" t="n">
+      <c r="M110" t="n">
         <v>-16</v>
       </c>
-      <c r="N111" t="n">
+      <c r="N110" t="n">
         <v>-1200</v>
       </c>
-      <c r="O111" t="n">
-        <v>4</v>
-      </c>
-      <c r="P111" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q111" t="inlineStr">
+      <c r="O110" t="n">
+        <v>4</v>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8795,68 +8720,68 @@
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" t="n">
+    <row r="111">
+      <c r="A111" t="n">
         <v>111</v>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B111" t="inlineStr">
         <is>
           <t>2026-06-05 11:02:13</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="D111" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E112" t="n">
+      <c r="E111" t="n">
         <v>23475.2</v>
       </c>
-      <c r="F112" t="n">
+      <c r="F111" t="n">
         <v>23408.5</v>
       </c>
-      <c r="G112" t="n">
+      <c r="G111" t="n">
         <v>23541.9</v>
       </c>
-      <c r="H112" t="n">
+      <c r="H111" t="n">
         <v>66.7</v>
       </c>
-      <c r="I112" t="n">
+      <c r="I111" t="n">
         <v>66.7</v>
       </c>
-      <c r="J112" t="inlineStr">
+      <c r="J111" t="inlineStr">
         <is>
           <t>2026-06-05 11:05:56</t>
         </is>
       </c>
-      <c r="K112" t="n">
+      <c r="K111" t="n">
         <v>23545</v>
       </c>
-      <c r="L112" t="inlineStr">
+      <c r="L111" t="inlineStr">
         <is>
           <t>TARGET_HIT</t>
         </is>
       </c>
-      <c r="M112" t="n">
+      <c r="M111" t="n">
         <v>69.8</v>
       </c>
-      <c r="N112" t="n">
+      <c r="N111" t="n">
         <v>5235</v>
       </c>
-      <c r="O112" t="n">
-        <v>4</v>
-      </c>
-      <c r="P112" t="inlineStr">
+      <c r="O111" t="n">
+        <v>4</v>
+      </c>
+      <c r="P111" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q112" t="inlineStr">
+      <c r="Q111" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8870,68 +8795,68 @@
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" t="n">
+    <row r="112">
+      <c r="A112" t="n">
         <v>112</v>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B112" t="inlineStr">
         <is>
           <t>2026-06-05 11:10:25</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D112" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E113" t="n">
+      <c r="E112" t="n">
         <v>23569.3</v>
       </c>
-      <c r="F113" t="n">
+      <c r="F112" t="n">
         <v>23502.6</v>
       </c>
-      <c r="G113" t="n">
+      <c r="G112" t="n">
         <v>23636</v>
       </c>
-      <c r="H113" t="n">
+      <c r="H112" t="n">
         <v>66.7</v>
       </c>
-      <c r="I113" t="n">
+      <c r="I112" t="n">
         <v>66.7</v>
       </c>
-      <c r="J113" t="inlineStr">
+      <c r="J112" t="inlineStr">
         <is>
           <t>2026-06-05 11:14:18</t>
         </is>
       </c>
-      <c r="K113" t="n">
+      <c r="K112" t="n">
         <v>23537.9</v>
       </c>
-      <c r="L113" t="inlineStr">
+      <c r="L112" t="inlineStr">
         <is>
           <t>COUNTER_VIEW_FLIP</t>
         </is>
       </c>
-      <c r="M113" t="n">
+      <c r="M112" t="n">
         <v>-31.4</v>
       </c>
-      <c r="N113" t="n">
+      <c r="N112" t="n">
         <v>-2355</v>
       </c>
-      <c r="O113" t="n">
-        <v>4</v>
-      </c>
-      <c r="P113" t="inlineStr">
+      <c r="O112" t="n">
+        <v>4</v>
+      </c>
+      <c r="P112" t="inlineStr">
         <is>
           <t>BULLISH</t>
         </is>
       </c>
-      <c r="Q113" t="inlineStr">
+      <c r="Q112" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -8945,68 +8870,68 @@
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" t="n">
+    <row r="113">
+      <c r="A113" t="n">
         <v>113</v>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B113" t="inlineStr">
         <is>
           <t>2026-06-05 11:14:20</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
         <is>
           <t>NSE:NIFTY26JUNFUT</t>
         </is>
       </c>
-      <c r="E114" t="n">
+      <c r="E113" t="n">
         <v>23539.8</v>
       </c>
-      <c r="F114" t="n">
+      <c r="F113" t="n">
         <v>23606.5</v>
       </c>
-      <c r="G114" t="n">
+      <c r="G113" t="n">
         <v>23473.1</v>
       </c>
-      <c r="H114" t="n">
+      <c r="H113" t="n">
         <v>66.7</v>
       </c>
-      <c r="I114" t="n">
+      <c r="I113" t="n">
         <v>66.7</v>
       </c>
-      <c r="J114" t="inlineStr">
+      <c r="J113" t="inlineStr">
         <is>
           <t>2026-06-05 11:21:11</t>
         </is>
       </c>
-      <c r="K114" t="n">
+      <c r="K113" t="n">
         <v>23471</v>
       </c>
-      <c r="L114" t="inlineStr">
+      <c r="L113" t="inlineStr">
         <is>
           <t>TARGET_HIT</t>
         </is>
       </c>
-      <c r="M114" t="n">
+      <c r="M113" t="n">
         <v>68.8</v>
       </c>
-      <c r="N114" t="n">
+      <c r="N113" t="n">
         <v>5160</v>
       </c>
-      <c r="O114" t="n">
-        <v>4</v>
-      </c>
-      <c r="P114" t="inlineStr">
-        <is>
-          <t>BEARISH</t>
-        </is>
-      </c>
-      <c r="Q114" t="inlineStr">
+      <c r="O113" t="n">
+        <v>4</v>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ──────────────────────────────
@@ -9041,8 +8966,8 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -14664,7 +14589,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
@@ -14684,7 +14609,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
@@ -14695,7 +14620,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>38.05%</t>
+          <t>38.39%</t>
         </is>
       </c>
     </row>
@@ -14707,7 +14632,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 9,562.50</t>
+          <t>Rs. 23,482.50</t>
         </is>
       </c>
     </row>
@@ -14719,7 +14644,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>127.50</t>
+          <t>313.10</t>
         </is>
       </c>
     </row>
@@ -14743,7 +14668,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -2,256.96</t>
+          <t>Rs. -2,087.93</t>
         </is>
       </c>
     </row>
@@ -14767,7 +14692,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rs. -13,920.00</t>
+          <t>Rs. -6,540.00</t>
         </is>
       </c>
     </row>
@@ -14779,7 +14704,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.16</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14726,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-06 20:17:36</t>
+          <t>2026-06-06 22:33:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 08-06-2026 11:54:17.84
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q113"/>
+  <dimension ref="A1:Q115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -435,7 +435,7 @@
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
@@ -8941,6 +8941,172 @@
   ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
   ✅ 4. Order Flow: Sell dominant (0.0x)
   🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>114</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-06-08 09:58:36</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>23266.1</v>
+      </c>
+      <c r="F114" t="n">
+        <v>23199.4</v>
+      </c>
+      <c r="G114" t="n">
+        <v>23332.8</v>
+      </c>
+      <c r="H114" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I114" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:07:16</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>23225.2</v>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>-40.9</v>
+      </c>
+      <c r="N114" t="n">
+        <v>-3067.5</v>
+      </c>
+      <c r="O114" t="n">
+        <v>4</v>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 1.11 → 1.14 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23200: CE 5m -420,160 | PE 5m +993,200 | OTM CE -166,530 | OTM PE +958,945
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (40.6x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────
+──────────────────────────────
+🤖 KRONOS PRICE FORECAST (non-binding)
+  Direction : BULLISH
+  Δ Predicted: +169.7 pts over next 25 min
+  Confidence: HIGH
+  Signal    : ✅ AGREES with trade
+  Updated   : 09:57:14
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>115</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-06-08 10:07:17</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>23230</v>
+      </c>
+      <c r="F115" t="n">
+        <v>23296.7</v>
+      </c>
+      <c r="G115" t="n">
+        <v>23163.3</v>
+      </c>
+      <c r="H115" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I115" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>2026-06-08 11:39:52</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>23264</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M115" t="n">
+        <v>-34</v>
+      </c>
+      <c r="N115" t="n">
+        <v>-2550</v>
+      </c>
+      <c r="O115" t="n">
+        <v>4</v>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.32 → 1.31 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23150: CE 5m +71,370 | PE 5m -260,390 | OTM CE +826,410 | OTM PE -883,675
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────
+──────────────────────────────
+🤖 KRONOS PRICE FORECAST (non-binding)
+  Direction : BULLISH
+  Δ Predicted: +126.4 pts over next 25 min
+  Confidence: HIGH
+  Signal    : ⚠️ CONFLICTS with trade
+  Updated   : 10:06:28
 ──────────────────────────────</t>
         </is>
       </c>
@@ -14589,7 +14755,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3">
@@ -14609,7 +14775,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5">
@@ -14620,7 +14786,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>38.39%</t>
+          <t>37.72%</t>
         </is>
       </c>
     </row>
@@ -14632,7 +14798,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 23,482.50</t>
+          <t>Rs. 17,865.00</t>
         </is>
       </c>
     </row>
@@ -14644,7 +14810,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>313.10</t>
+          <t>238.20</t>
         </is>
       </c>
     </row>
@@ -14668,7 +14834,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -2,087.93</t>
+          <t>Rs. -2,108.24</t>
         </is>
       </c>
     </row>
@@ -14704,7 +14870,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.12</t>
         </is>
       </c>
     </row>
@@ -14726,7 +14892,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-08 09:44:17</t>
+          <t>2026-06-08 11:49:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 08-06-2026 15:30:31.67
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q115"/>
+  <dimension ref="A1:Q117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9111,6 +9111,172 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>116</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-06-08 11:39:53</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>23264</v>
+      </c>
+      <c r="F116" t="n">
+        <v>23197.3</v>
+      </c>
+      <c r="G116" t="n">
+        <v>23330.7</v>
+      </c>
+      <c r="H116" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I116" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>2026-06-08 12:05:54</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>23265</v>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M116" t="n">
+        <v>1</v>
+      </c>
+      <c r="N116" t="n">
+        <v>75</v>
+      </c>
+      <c r="O116" t="n">
+        <v>4</v>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Rising 1.17 → 1.17 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23200: CE 5m +3,250 | PE 5m +190,125 | OTM CE +22,425 | OTM PE +184,210
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (24.2x)
+  🟢🟢 ALL 4 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────
+──────────────────────────────
+🤖 KRONOS PRICE FORECAST (non-binding)
+  Direction : BULLISH
+  Δ Predicted: +24.0 pts over next 25 min
+  Confidence: HIGH
+  Signal    : ✅ AGREES with trade
+  Updated   : 11:39:04
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>117</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-06-08 12:05:55</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>23265</v>
+      </c>
+      <c r="F117" t="n">
+        <v>23331.7</v>
+      </c>
+      <c r="G117" t="n">
+        <v>23198.3</v>
+      </c>
+      <c r="H117" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I117" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>2026-06-08 12:51:07</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>23334</v>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M117" t="n">
+        <v>-69</v>
+      </c>
+      <c r="N117" t="n">
+        <v>-5175</v>
+      </c>
+      <c r="O117" t="n">
+        <v>4</v>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (4/4)
+  ✅ 1. PCR Trend: PCR Falling 1.25 → 1.25 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23200: CE 5m +220,740 | PE 5m +145,990 | OTM CE +148,980 | OTM PE -67,860
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  🔴🔴 ALL 4 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────
+──────────────────────────────
+🤖 KRONOS PRICE FORECAST (non-binding)
+  Direction : BEARISH
+  Δ Predicted: -23.4 pts over next 25 min
+  Confidence: HIGH
+  Signal    : ✅ AGREES with trade
+  Updated   : 12:05:50
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9122,7 +9288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O118"/>
+  <dimension ref="A1:O122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -14718,6 +14884,194 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>170</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:01:45</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>4</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G119" t="n">
+        <v>23324.2</v>
+      </c>
+      <c r="H119" t="n">
+        <v>23390.9</v>
+      </c>
+      <c r="I119" t="n">
+        <v>23257.5</v>
+      </c>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>171</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:16:52</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>4</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>23220</v>
+      </c>
+      <c r="H120" t="n">
+        <v>23286.7</v>
+      </c>
+      <c r="I120" t="n">
+        <v>23153.3</v>
+      </c>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>172</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:24:07</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>4</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>23202.3</v>
+      </c>
+      <c r="H121" t="n">
+        <v>23269</v>
+      </c>
+      <c r="I121" t="n">
+        <v>23135.6</v>
+      </c>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>173</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-06-08 14:39:08</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>DAILY_LOSS_LIMIT_REACHED</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>4</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="G122" t="n">
+        <v>23210</v>
+      </c>
+      <c r="H122" t="n">
+        <v>23276.7</v>
+      </c>
+      <c r="I122" t="n">
+        <v>23143.3</v>
+      </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14755,7 +15109,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3">
@@ -14765,7 +15119,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4">
@@ -14775,7 +15129,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
@@ -14786,7 +15140,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>37.72%</t>
+          <t>37.93%</t>
         </is>
       </c>
     </row>
@@ -14798,7 +15152,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 17,865.00</t>
+          <t>Rs. 12,765.00</t>
         </is>
       </c>
     </row>
@@ -14810,7 +15164,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>238.20</t>
+          <t>170.20</t>
         </is>
       </c>
     </row>
@@ -14822,7 +15176,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs. 3,896.51</t>
+          <t>Rs. 3,809.66</t>
         </is>
       </c>
     </row>
@@ -14834,7 +15188,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -2,108.24</t>
+          <t>Rs. -2,150.83</t>
         </is>
       </c>
     </row>
@@ -14870,7 +15224,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.08</t>
         </is>
       </c>
     </row>
@@ -14881,7 +15235,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14">
@@ -14892,7 +15246,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-08 11:49:11</t>
+          <t>2026-06-08 15:26:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 09-06-2026 15:49:35.84
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q117"/>
+  <dimension ref="A1:Q119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9273,6 +9273,158 @@
   Confidence: HIGH
   Signal    : ✅ AGREES with trade
   Updated   : 12:05:50
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>118</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:06:26</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>23226.8</v>
+      </c>
+      <c r="F118" t="n">
+        <v>23160.1</v>
+      </c>
+      <c r="G118" t="n">
+        <v>23293.5</v>
+      </c>
+      <c r="H118" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I118" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>2026-06-09 14:39:34</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>23294</v>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M118" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="N118" t="n">
+        <v>5040</v>
+      </c>
+      <c r="O118" t="n">
+        <v>5</v>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Rising 0.76 → 0.76 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23200: CE 5m -2,282,085 | PE 5m +2,054,455 | OTM CE -873,925 | OTM PE +2,525,380
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (49.5x)
+  ✅ 5. Kronos Forecast: BULLISH (+58.5 pts | HIGH confidence)
+  🟢🟢 ALL 5 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>119</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-06-09 14:41:15</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>23313</v>
+      </c>
+      <c r="F119" t="n">
+        <v>23246.3</v>
+      </c>
+      <c r="G119" t="n">
+        <v>23379.7</v>
+      </c>
+      <c r="H119" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I119" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>2026-06-09 15:10:01</t>
+        </is>
+      </c>
+      <c r="K119" t="n">
+        <v>23337.9</v>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>EOD_CLOSE</t>
+        </is>
+      </c>
+      <c r="M119" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="N119" t="n">
+        <v>1867.5</v>
+      </c>
+      <c r="O119" t="n">
+        <v>5</v>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Rising 0.82 → 0.87 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (3/3) — ATM 23250: CE 5m -14,869,270 | PE 5m +9,249,435 | OTM CE +1,609,920 | OTM PE +2,020,720
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (21.5x)
+  ✅ 5. Kronos Forecast: BULLISH (+230.9 pts | HIGH confidence)
+  🟢🟢 ALL 5 CHECKS BULLISH — TRADE ENTRY
 ──────────────────────────────</t>
         </is>
       </c>
@@ -15109,7 +15261,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3">
@@ -15119,7 +15271,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4">
@@ -15140,7 +15292,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>37.93%</t>
+          <t>38.98%</t>
         </is>
       </c>
     </row>
@@ -15152,7 +15304,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 12,765.00</t>
+          <t>Rs. 19,672.50</t>
         </is>
       </c>
     </row>
@@ -15164,7 +15316,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>170.20</t>
+          <t>262.30</t>
         </is>
       </c>
     </row>
@@ -15176,7 +15328,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs. 3,809.66</t>
+          <t>Rs. 3,794.18</t>
         </is>
       </c>
     </row>
@@ -15224,7 +15376,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.13</t>
         </is>
       </c>
     </row>
@@ -15246,7 +15398,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-08 15:41:20</t>
+          <t>2026-06-09 15:45:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 10-06-2026 15:38:45.63
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q119"/>
+  <dimension ref="A1:Q123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9425,6 +9425,310 @@
   ✅ 4. Order Flow: Buy dominant (21.5x)
   ✅ 5. Kronos Forecast: BULLISH (+230.9 pts | HIGH confidence)
   🟢🟢 ALL 5 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>120</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-06-10 09:40:37</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>23369</v>
+      </c>
+      <c r="F120" t="n">
+        <v>23302.3</v>
+      </c>
+      <c r="G120" t="n">
+        <v>23435.7</v>
+      </c>
+      <c r="H120" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I120" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>2026-06-10 10:20:49</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>23352</v>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>COUNTER_VIEW_FLIP</t>
+        </is>
+      </c>
+      <c r="M120" t="n">
+        <v>-17</v>
+      </c>
+      <c r="N120" t="n">
+        <v>-1275</v>
+      </c>
+      <c r="O120" t="n">
+        <v>5</v>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Rising 1.10 → 1.11 (Bullish momentum)
+  ✅ 2. Near-Strike OI: Bullish (2/3) — ATM 23350: CE 5m +71,890 | PE 5m +507,650 | OTM CE +184,275 | OTM PE +574,015
+  ✅ 3. AI Timeframe Bias: 5m: BULLISH | 15m: BULLISH | 30m: BULLISH
+  ✅ 4. Order Flow: Buy dominant (27.3x)
+  ✅ 5. Kronos Forecast: BULLISH (+14.5 pts | MEDIUM confidence)
+  🟢🟢 ALL 5 CHECKS BULLISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>121</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-06-10 10:20:50</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>23355</v>
+      </c>
+      <c r="F121" t="n">
+        <v>23421.7</v>
+      </c>
+      <c r="G121" t="n">
+        <v>23288.3</v>
+      </c>
+      <c r="H121" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I121" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>2026-06-10 11:27:20</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>23425</v>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M121" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N121" t="n">
+        <v>-5250</v>
+      </c>
+      <c r="O121" t="n">
+        <v>5</v>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Falling 1.11 → 1.01 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23350: CE 5m +435,630 | PE 5m -391,950 | OTM CE +343,785 | OTM PE -364,650
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  ✅ 5. Kronos Forecast: BEARISH (-38.0 pts | HIGH confidence)
+  🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>122</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:11:45</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>23417</v>
+      </c>
+      <c r="F122" t="n">
+        <v>23483.7</v>
+      </c>
+      <c r="G122" t="n">
+        <v>23350.3</v>
+      </c>
+      <c r="H122" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I122" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:11:44</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>23350</v>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M122" t="n">
+        <v>67</v>
+      </c>
+      <c r="N122" t="n">
+        <v>5025</v>
+      </c>
+      <c r="O122" t="n">
+        <v>5</v>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Falling 1.18 → 1.18 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23400: CE 5m +173,095 | PE 5m -60,645 | OTM CE +36,660 | OTM PE -31,265
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  ✅ 5. Kronos Forecast: BEARISH (-77.2 pts | HIGH confidence)
+  🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>123</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:24:18</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>23349.9</v>
+      </c>
+      <c r="F123" t="n">
+        <v>23416.6</v>
+      </c>
+      <c r="G123" t="n">
+        <v>23283.2</v>
+      </c>
+      <c r="H123" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I123" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>2026-06-10 14:42:58</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>23275</v>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M123" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="N123" t="n">
+        <v>5617.5</v>
+      </c>
+      <c r="O123" t="n">
+        <v>5</v>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Falling 0.90 → 0.90 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23350: CE 5m +223,015 | PE 5m +28,145 | OTM CE +154,960 | OTM PE +38,610
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.1x)
+  ✅ 5. Kronos Forecast: BEARISH (-28.7 pts | HIGH confidence)
+  🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
 ──────────────────────────────</t>
         </is>
       </c>
@@ -15261,7 +15565,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3">
@@ -15271,7 +15575,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -15281,7 +15585,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5">
@@ -15292,7 +15596,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>38.98%</t>
+          <t>39.34%</t>
         </is>
       </c>
     </row>
@@ -15304,7 +15608,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 19,672.50</t>
+          <t>Rs. 23,790.00</t>
         </is>
       </c>
     </row>
@@ -15316,7 +15620,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>262.30</t>
+          <t>317.20</t>
         </is>
       </c>
     </row>
@@ -15328,7 +15632,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs. 3,794.18</t>
+          <t>Rs. 3,857.81</t>
         </is>
       </c>
     </row>
@@ -15340,7 +15644,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -2,150.83</t>
+          <t>Rs. -2,180.88</t>
         </is>
       </c>
     </row>
@@ -15376,7 +15680,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.15</t>
         </is>
       </c>
     </row>
@@ -15398,7 +15702,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-09 15:45:46</t>
+          <t>2026-06-10 15:30:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 11-06-2026 15:46:18.78
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q123"/>
+  <dimension ref="A1:Q124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9728,6 +9728,82 @@
   ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
   ✅ 4. Order Flow: Sell dominant (0.1x)
   ✅ 5. Kronos Forecast: BEARISH (-28.7 pts | HIGH confidence)
+  🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>124</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-06-11 13:46:12</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>23255</v>
+      </c>
+      <c r="F124" t="n">
+        <v>23321.7</v>
+      </c>
+      <c r="G124" t="n">
+        <v>23188.3</v>
+      </c>
+      <c r="H124" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I124" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>2026-06-11 15:01:12</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>23188.3</v>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="M124" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="N124" t="n">
+        <v>5002.5</v>
+      </c>
+      <c r="O124" t="n">
+        <v>5</v>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Falling 1.47 → 1.47 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23200: CE 5m +24,375 | PE 5m -40,755 | OTM CE +71,175 | OTM PE -56,095
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  ✅ 5. Kronos Forecast: BEARISH (-11.7 pts | MEDIUM confidence)
   🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
 ──────────────────────────────</t>
         </is>
@@ -15565,7 +15641,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3">
@@ -15575,7 +15651,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -15596,7 +15672,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>39.34%</t>
+          <t>39.84%</t>
         </is>
       </c>
     </row>
@@ -15608,7 +15684,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 23,790.00</t>
+          <t>Rs. 28,792.50</t>
         </is>
       </c>
     </row>
@@ -15620,7 +15696,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>317.20</t>
+          <t>383.90</t>
         </is>
       </c>
     </row>
@@ -15632,7 +15708,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs. 3,857.81</t>
+          <t>Rs. 3,881.17</t>
         </is>
       </c>
     </row>
@@ -15680,7 +15756,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.18</t>
         </is>
       </c>
     </row>
@@ -15702,7 +15778,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-10 15:39:46</t>
+          <t>2026-06-11 15:44:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and Excel files - 12-06-2026 16:58:42.28
</commit_message>
<xml_diff>
--- a/paper_trades_analysis.xlsx
+++ b/paper_trades_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q124"/>
+  <dimension ref="A1:Q127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -436,7 +436,7 @@
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
@@ -9804,6 +9804,234 @@
   ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
   ✅ 4. Order Flow: Sell dominant (0.0x)
   ✅ 5. Kronos Forecast: BEARISH (-11.7 pts | MEDIUM confidence)
+  🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>125</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:49:21</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>23344</v>
+      </c>
+      <c r="F125" t="n">
+        <v>23410.7</v>
+      </c>
+      <c r="G125" t="n">
+        <v>23277.3</v>
+      </c>
+      <c r="H125" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I125" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>2026-06-12 13:27:02</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>23417.4</v>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M125" t="n">
+        <v>-73.40000000000001</v>
+      </c>
+      <c r="N125" t="n">
+        <v>-5505</v>
+      </c>
+      <c r="O125" t="n">
+        <v>5</v>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Falling 0.81 → 0.81 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (3/3) — ATM 23300: CE 5m +1,044,680 | PE 5m -86,255 | OTM CE +853,320 | OTM PE -525,525
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  ✅ 5. Kronos Forecast: BEARISH (-64.0 pts | HIGH confidence)
+  🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>126</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-06-12 14:40:24</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>23624.1</v>
+      </c>
+      <c r="F126" t="n">
+        <v>23690.8</v>
+      </c>
+      <c r="G126" t="n">
+        <v>23557.4</v>
+      </c>
+      <c r="H126" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I126" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>2026-06-12 15:03:10</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>23693</v>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="M126" t="n">
+        <v>-68.90000000000001</v>
+      </c>
+      <c r="N126" t="n">
+        <v>-5167.5</v>
+      </c>
+      <c r="O126" t="n">
+        <v>5</v>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Falling 1.18 → 1.17 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23550: CE 5m +256,815 | PE 5m -35,685 | OTM CE -22,425 | OTM PE +32,890
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  ✅ 5. Kronos Forecast: BEARISH (-301.1 pts | HIGH confidence)
+  🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
+──────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>127</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-06-12 15:05:09</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>NSE:NIFTY26JUNFUT</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>23699.5</v>
+      </c>
+      <c r="F127" t="n">
+        <v>23766.2</v>
+      </c>
+      <c r="G127" t="n">
+        <v>23632.8</v>
+      </c>
+      <c r="H127" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I127" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>2026-06-12 15:10:03</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>23680</v>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>EOD_CLOSE</t>
+        </is>
+      </c>
+      <c r="M127" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="N127" t="n">
+        <v>1462.5</v>
+      </c>
+      <c r="O127" t="n">
+        <v>5</v>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+──────────────────────────────
+🎯 INSTITUTIONAL CHECKLIST (5/5)
+  ✅ 1. PCR Trend: PCR Falling 1.13 → 1.11 (Bearish momentum)
+  ✅ 2. Near-Strike OI: Bearish (2/3) — ATM 23650: CE 5m +37,440 | PE 5m -40,040 | OTM CE -775,580 | OTM PE -31,720
+  ✅ 3. AI Timeframe Bias: 5m: BEARISH | 15m: BEARISH | 30m: BEARISH
+  ✅ 4. Order Flow: Sell dominant (0.0x)
+  ✅ 5. Kronos Forecast: BEARISH (-281.9 pts | HIGH confidence)
   🔴🔴 ALL 5 CHECKS BEARISH — TRADE ENTRY
 ──────────────────────────────</t>
         </is>
@@ -15641,7 +15869,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3">
@@ -15651,7 +15879,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -15661,7 +15889,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
@@ -15672,7 +15900,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>39.84%</t>
+          <t>39.68%</t>
         </is>
       </c>
     </row>
@@ -15684,7 +15912,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rs. 28,792.50</t>
+          <t>Rs. 19,582.50</t>
         </is>
       </c>
     </row>
@@ -15696,7 +15924,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>383.90</t>
+          <t>261.10</t>
         </is>
       </c>
     </row>
@@ -15708,7 +15936,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rs. 3,881.17</t>
+          <t>Rs. 3,832.80</t>
         </is>
       </c>
     </row>
@@ -15720,7 +15948,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rs. -2,180.88</t>
+          <t>Rs. -2,263.91</t>
         </is>
       </c>
     </row>
@@ -15756,7 +15984,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.11</t>
         </is>
       </c>
     </row>
@@ -15778,7 +16006,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-11 15:44:04</t>
+          <t>2026-06-12 16:56:38</t>
         </is>
       </c>
     </row>

</xml_diff>